<commit_message>
Readiness tool: print-safe build (no embedded chart, data bars, rich text or sheet protection)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
@@ -30,12 +30,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0&quot; / 4&quot;"/>
-    <numFmt numFmtId="165" formatCode=";;;"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,6 +100,10 @@
       <b val="1"/>
       <color rgb="004F2D7F"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -208,9 +211,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00000000"/>
-      <sz val="7.5"/>
+      <color rgb="004F2D7F"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -411,46 +413,46 @@
   </cellStyleXfs>
   <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -475,19 +477,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -502,7 +504,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -512,69 +514,69 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -583,72 +585,72 @@
     <xf numFmtId="9" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="30" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -827,146 +829,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <plotArea>
-      <radarChart>
-        <radarStyle val="marker"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <v>Current readiness (%)</v>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
-              <a:solidFill>
-                <a:srgbClr val="4F2D7F"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="4F2D7F"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Calc'!$H$37:$H$43</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Calc'!$I$37:$I$43</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>Target - Repeatable (70%)</v>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="00A7B5"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Calc'!$H$37:$H$43</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Calc'!$J$37:$J$43</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </radarChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <max val="100"/>
-          <min val="0"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <majorUnit val="25"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>16</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3348000" cy="3096000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1843,22 +1705,8 @@
       </c>
       <c r="D10" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Which statement best describes how AI is used in your organisation today (including AI embedded in software and tools used by staff)?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Consider approved and unapproved tools, vendor software with AI features and AI used by suppliers on your behalf.</t>
-          </r>
+          <t>Which statement best describes how AI is used in your organisation today (including AI embedded in software and tools used by staff)?
+Guidance: Consider approved and unapproved tools, vendor software with AI features and AI used by suppliers on your behalf.</t>
         </is>
       </c>
       <c r="E10" s="33" t="n"/>
@@ -1902,22 +1750,8 @@
       </c>
       <c r="D11" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>What is the most significant type of decision or outcome your AI systems influence?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Answer for the highest-impact AI use case in scope (AIAF: 'worst credible harm').</t>
-          </r>
+          <t>What is the most significant type of decision or outcome your AI systems influence?
+Guidance: Answer for the highest-impact AI use case in scope (AIAF: 'worst credible harm').</t>
         </is>
       </c>
       <c r="E11" s="33" t="n"/>
@@ -1961,22 +1795,8 @@
       </c>
       <c r="D12" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>What is the most sensitive data processed by your AI systems (including data staff enter into AI tools)?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Include prompts, uploaded documents, training / fine-tuning data, retrieval sources and logs.</t>
-          </r>
+          <t>What is the most sensitive data processed by your AI systems (including data staff enter into AI tools)?
+Guidance: Include prompts, uploaded documents, training / fine-tuning data, retrieval sources and logs.</t>
         </is>
       </c>
       <c r="E12" s="33" t="n"/>
@@ -2020,22 +1840,8 @@
       </c>
       <c r="D13" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>How much human oversight applies to AI outputs, and how reversible are the outcomes?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-AIAF considers autonomy, human oversight and whether outputs are reversible or correctable.</t>
-          </r>
+          <t>How much human oversight applies to AI outputs, and how reversible are the outcomes?
+Guidance: AIAF considers autonomy, human oversight and whether outputs are reversible or correctable.</t>
         </is>
       </c>
       <c r="E13" s="33" t="n"/>
@@ -2095,22 +1901,8 @@
       </c>
       <c r="D15" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is there executive ownership and an approved AI strategy that defines the ambition, where AI will be used and the organisation's AI risk appetite?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: approved AI strategy, named executive sponsor, risk appetite statement, experimentation boundaries.</t>
-          </r>
+          <t>Is there executive ownership and an approved AI strategy that defines the ambition, where AI will be used and the organisation's AI risk appetite?
+Guidance: Evidence: approved AI strategy, named executive sponsor, risk appetite statement, experimentation boundaries.</t>
         </is>
       </c>
       <c r="E15" s="33" t="n"/>
@@ -2155,22 +1947,8 @@
       </c>
       <c r="D16" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>How are AI use cases identified, prioritised, approved and measured for value?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: intake form, prioritisation criteria, business cases, benefit KPIs, portfolio reviews.</t>
-          </r>
+          <t>How are AI use cases identified, prioritised, approved and measured for value?
+Guidance: Evidence: intake form, prioritisation criteria, business cases, benefit KPIs, portfolio reviews.</t>
         </is>
       </c>
       <c r="E16" s="33" t="n"/>
@@ -2215,22 +1993,8 @@
       </c>
       <c r="D17" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Do you have an approved AI (acceptable-use) policy and a process to identify and comply with applicable AI-related regulation (e.g., Bahrain PDPL, CBB rules, EU AI Act)?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI policy, approved-tools list, staff acknowledgements, obligations register, compliance reviews.</t>
-          </r>
+          <t>Do you have an approved AI (acceptable-use) policy and a process to identify and comply with applicable AI-related regulation (e.g., Bahrain PDPL, CBB rules, EU AI Act)?
+Guidance: Evidence: AI policy, approved-tools list, staff acknowledgements, obligations register, compliance reviews.</t>
         </is>
       </c>
       <c r="E17" s="33" t="n"/>
@@ -2275,22 +2039,8 @@
       </c>
       <c r="D18" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Do you maintain an inventory of AI systems with named owners, and assess AI risks and impacts (including third-party AI) before and after deployment?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI register, risk-tiering records, impact assessments, vendor AI due diligence, re-assessment records.</t>
-          </r>
+          <t>Do you maintain an inventory of AI systems with named owners, and assess AI risks and impacts (including third-party AI) before and after deployment?
+Guidance: Evidence: AI register, risk-tiering records, impact assessments, vendor AI due diligence, re-assessment records.</t>
         </is>
       </c>
       <c r="E18" s="33" t="n"/>
@@ -2335,22 +2085,8 @@
       </c>
       <c r="D19" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are there practical guardrails for fairness, transparency and human oversight, overseen by an AI committee or centre of excellence?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: committee / CoE charter, guardrail standards, human-in-charge procedures, bias tests, AI disclosures, appeal routes.</t>
-          </r>
+          <t>Are there practical guardrails for fairness, transparency and human oversight, overseen by an AI committee or centre of excellence?
+Guidance: Evidence: committee / CoE charter, guardrail standards, human-in-charge procedures, bias tests, AI disclosures, appeal routes.</t>
         </is>
       </c>
       <c r="E19" s="33" t="n"/>
@@ -2395,22 +2131,8 @@
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Have staff received AI literacy training appropriate to their role, and are specialist AI, governance and security skills being developed?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: training curricula, completion records, role-based pathways, deepfake / phishing simulations, workforce plan.</t>
-          </r>
+          <t>Have staff received AI literacy training appropriate to their role, and are specialist AI, governance and security skills being developed?
+Guidance: Evidence: training curricula, completion records, role-based pathways, deepfake / phishing simulations, workforce plan.</t>
         </is>
       </c>
       <c r="E20" s="33" t="n"/>
@@ -2455,22 +2177,8 @@
       </c>
       <c r="D21" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is data used by AI classified, quality-assured, traceable and protected in line with privacy requirements (e.g., Bahrain PDPL)?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: data classification applied to AI, data-readiness assessments, lineage, DPIAs, redaction / anonymisation, transfer assessments.</t>
-          </r>
+          <t>Is data used by AI classified, quality-assured, traceable and protected in line with privacy requirements (e.g., Bahrain PDPL)?
+Guidance: Evidence: data classification applied to AI, data-readiness assessments, lineage, DPIAs, redaction / anonymisation, transfer assessments.</t>
         </is>
       </c>
       <c r="E21" s="33" t="n"/>
@@ -2515,22 +2223,8 @@
       </c>
       <c r="D22" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is there a common AI reference architecture with standard integration patterns, and are AI systems monitored for performance, drift and cost?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: reference architecture, approved platforms, integration / agent patterns, monitoring dashboards, cost reports.</t>
-          </r>
+          <t>Is there a common AI reference architecture with standard integration patterns, and are AI systems monitored for performance, drift and cost?
+Guidance: Evidence: reference architecture, approved platforms, integration / agent patterns, monitoring dashboards, cost reports.</t>
         </is>
       </c>
       <c r="E22" s="33" t="n"/>
@@ -2575,22 +2269,8 @@
       </c>
       <c r="D23" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are AI systems protected with least-privilege access, secure development and testing (incl. red teaming for prompt injection), and runtime logging?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI threat models, access reviews (incl. agent identities), AI red-team reports, guardrail and sandbox configurations, audit logs. Detailed test: GT AI Security &amp; Agent Audit Checklist.</t>
-          </r>
+          <t>Are AI systems protected with least-privilege access, secure development and testing (incl. red teaming for prompt injection), and runtime logging?
+Guidance: Evidence: AI threat models, access reviews (incl. agent identities), AI red-team reports, guardrail and sandbox configurations, audit logs. Detailed test: GT AI Security &amp; Agent Audit Checklist.</t>
         </is>
       </c>
       <c r="E23" s="33" t="n"/>
@@ -2635,22 +2315,8 @@
       </c>
       <c r="D24" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is the organisation prepared for AI-enabled attacks such as deepfake impersonation, AI-crafted phishing and automated exploitation?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI threat intelligence, out-of-band verification procedures, deepfake simulations, SOC use cases, playbooks, patch metrics.</t>
-          </r>
+          <t>Is the organisation prepared for AI-enabled attacks such as deepfake impersonation, AI-crafted phishing and automated exploitation?
+Guidance: Evidence: AI threat intelligence, out-of-band verification procedures, deepfake simulations, SOC use cases, playbooks, patch metrics.</t>
         </is>
       </c>
       <c r="E24" s="33" t="n"/>
@@ -2695,22 +2361,8 @@
       </c>
       <c r="D25" s="32" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are AI incidents detected, managed and reported, and is AI governance subject to internal audit or independent assurance?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI incident categories, notification criteria, incident logs, internal-audit reports, vendor assurance, certification status.</t>
-          </r>
+          <t>Are AI incidents detected, managed and reported, and is AI governance subject to internal audit or independent assurance?
+Guidance: Evidence: AI incident categories, notification criteria, incident logs, internal-audit reports, vendor assurance, certification status.</t>
         </is>
       </c>
       <c r="E25" s="33" t="n"/>
@@ -2742,7 +2394,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="16">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="D4"/>
@@ -3137,9 +2788,14 @@
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>Progress</t>
-        </is>
-      </c>
+          <t>Progress  (each block = 5%;  target 70% = 14 blocks)</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="21" t="n"/>
+      <c r="K17" s="21" t="n"/>
     </row>
     <row r="18" ht="25" customHeight="1">
       <c r="B18" s="56" t="inlineStr">
@@ -3157,9 +2813,14 @@
         <v/>
       </c>
       <c r="F18" s="57">
-        <f>IF(Calc!B37="",0,Calc!B37)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B37="","",REPT("■",ROUND(Calc!B37*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B37*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="21" t="n"/>
+      <c r="J18" s="21" t="n"/>
+      <c r="K18" s="21" t="n"/>
     </row>
     <row r="19" ht="25" customHeight="1">
       <c r="B19" s="56" t="inlineStr">
@@ -3177,9 +2838,14 @@
         <v/>
       </c>
       <c r="F19" s="57">
-        <f>IF(Calc!B38="",0,Calc!B38)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B38="","",REPT("■",ROUND(Calc!B38*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B38*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
     </row>
     <row r="20" ht="25" customHeight="1">
       <c r="B20" s="56" t="inlineStr">
@@ -3197,9 +2863,14 @@
         <v/>
       </c>
       <c r="F20" s="57">
-        <f>IF(Calc!B39="",0,Calc!B39)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B39="","",REPT("■",ROUND(Calc!B39*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B39*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G20" s="21" t="n"/>
+      <c r="H20" s="21" t="n"/>
+      <c r="I20" s="21" t="n"/>
+      <c r="J20" s="21" t="n"/>
+      <c r="K20" s="21" t="n"/>
     </row>
     <row r="21" ht="25" customHeight="1">
       <c r="B21" s="56" t="inlineStr">
@@ -3217,9 +2888,14 @@
         <v/>
       </c>
       <c r="F21" s="57">
-        <f>IF(Calc!B40="",0,Calc!B40)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B40="","",REPT("■",ROUND(Calc!B40*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B40*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G21" s="21" t="n"/>
+      <c r="H21" s="21" t="n"/>
+      <c r="I21" s="21" t="n"/>
+      <c r="J21" s="21" t="n"/>
+      <c r="K21" s="21" t="n"/>
     </row>
     <row r="22" ht="25" customHeight="1">
       <c r="B22" s="56" t="inlineStr">
@@ -3237,9 +2913,14 @@
         <v/>
       </c>
       <c r="F22" s="57">
-        <f>IF(Calc!B41="",0,Calc!B41)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B41="","",REPT("■",ROUND(Calc!B41*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B41*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G22" s="21" t="n"/>
+      <c r="H22" s="21" t="n"/>
+      <c r="I22" s="21" t="n"/>
+      <c r="J22" s="21" t="n"/>
+      <c r="K22" s="21" t="n"/>
     </row>
     <row r="23" ht="25" customHeight="1">
       <c r="B23" s="56" t="inlineStr">
@@ -3257,9 +2938,14 @@
         <v/>
       </c>
       <c r="F23" s="57">
-        <f>IF(Calc!B42="",0,Calc!B42)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B42="","",REPT("■",ROUND(Calc!B42*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B42*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="21" t="n"/>
+      <c r="K23" s="21" t="n"/>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="B24" s="56" t="inlineStr">
@@ -3277,9 +2963,14 @@
         <v/>
       </c>
       <c r="F24" s="57">
-        <f>IF(Calc!B43="",0,Calc!B43)</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B43="","",REPT("■",ROUND(Calc!B43*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B43*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="21" t="n"/>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="B25" s="58" t="inlineStr">
@@ -3297,9 +2988,14 @@
         <v/>
       </c>
       <c r="F25" s="60">
-        <f>"Target 70%"</f>
-        <v/>
-      </c>
+        <f>IF(Calc!B45="","",REPT("■",ROUND(Calc!B45*20,0))&amp;REPT("□",MAX(0,14-ROUND(Calc!B45*20,0))))</f>
+        <v/>
+      </c>
+      <c r="G25" s="21" t="n"/>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="21" t="n"/>
+      <c r="J25" s="21" t="n"/>
+      <c r="K25" s="21" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="B27" s="23" t="inlineStr">
@@ -5170,7 +4866,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="263">
     <mergeCell ref="B92:K92"/>
     <mergeCell ref="E118:G118"/>
@@ -5203,13 +4898,13 @@
     <mergeCell ref="B94:D94"/>
     <mergeCell ref="I59:K59"/>
     <mergeCell ref="B70:K70"/>
-    <mergeCell ref="F21"/>
     <mergeCell ref="G95:K95"/>
     <mergeCell ref="G58:H58"/>
     <mergeCell ref="I65:K65"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B120:K120"/>
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="F25:K25"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="H52:K52"/>
     <mergeCell ref="B33:C33"/>
@@ -5225,6 +4920,7 @@
     <mergeCell ref="G99:K99"/>
     <mergeCell ref="D57:F57"/>
     <mergeCell ref="G59:H59"/>
+    <mergeCell ref="F24:K24"/>
     <mergeCell ref="B98:D98"/>
     <mergeCell ref="J73:K73"/>
     <mergeCell ref="B25:C25"/>
@@ -5244,6 +4940,7 @@
     <mergeCell ref="H115:J115"/>
     <mergeCell ref="F89:J89"/>
     <mergeCell ref="B36:K36"/>
+    <mergeCell ref="F23:K23"/>
     <mergeCell ref="I62:K62"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="B11:C11"/>
@@ -5251,7 +4948,6 @@
     <mergeCell ref="G101:K101"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="F45:G45"/>
-    <mergeCell ref="F25"/>
     <mergeCell ref="F105:K105"/>
     <mergeCell ref="G62:H62"/>
     <mergeCell ref="I64:K64"/>
@@ -5266,15 +4962,15 @@
     <mergeCell ref="B110:D110"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F24"/>
     <mergeCell ref="G65:H65"/>
+    <mergeCell ref="B84:C84"/>
     <mergeCell ref="D60:F60"/>
-    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B100:D100"/>
     <mergeCell ref="J75:K75"/>
-    <mergeCell ref="B100:D100"/>
     <mergeCell ref="B109:D109"/>
     <mergeCell ref="H49:K49"/>
     <mergeCell ref="B47:D47"/>
+    <mergeCell ref="F19:K19"/>
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="F48:G48"/>
     <mergeCell ref="B46:D46"/>
@@ -5288,7 +4984,6 @@
     <mergeCell ref="H118:J118"/>
     <mergeCell ref="D89:E89"/>
     <mergeCell ref="K115"/>
-    <mergeCell ref="F23"/>
     <mergeCell ref="G60:H60"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="G9:H9"/>
@@ -5298,16 +4993,19 @@
     <mergeCell ref="E45"/>
     <mergeCell ref="D71"/>
     <mergeCell ref="G96:K96"/>
+    <mergeCell ref="F20:K20"/>
     <mergeCell ref="I66:K66"/>
     <mergeCell ref="D39:G39"/>
     <mergeCell ref="D34:K34"/>
     <mergeCell ref="B81:C81"/>
     <mergeCell ref="D81:E81"/>
+    <mergeCell ref="F17:K17"/>
     <mergeCell ref="H48:K48"/>
     <mergeCell ref="G98:K98"/>
     <mergeCell ref="B56:C56"/>
     <mergeCell ref="D38:G38"/>
     <mergeCell ref="B58:C58"/>
+    <mergeCell ref="F53:G53"/>
     <mergeCell ref="H117:J117"/>
     <mergeCell ref="I67:K67"/>
     <mergeCell ref="D11:K11"/>
@@ -5317,7 +5015,6 @@
     <mergeCell ref="D58:F58"/>
     <mergeCell ref="B113:K113"/>
     <mergeCell ref="B60:C60"/>
-    <mergeCell ref="F19"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="F50:G50"/>
     <mergeCell ref="B57:C57"/>
@@ -5340,7 +5037,6 @@
     <mergeCell ref="H116:J116"/>
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="I40:K40"/>
-    <mergeCell ref="F20"/>
     <mergeCell ref="D59:F59"/>
     <mergeCell ref="G64:H64"/>
     <mergeCell ref="B83:C83"/>
@@ -5372,6 +5068,7 @@
     <mergeCell ref="B42:G42"/>
     <mergeCell ref="B59:C59"/>
     <mergeCell ref="B101:D101"/>
+    <mergeCell ref="F18:K18"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="J72:K72"/>
     <mergeCell ref="F110:K110"/>
@@ -5387,6 +5084,7 @@
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="F109:K109"/>
     <mergeCell ref="E73:I73"/>
+    <mergeCell ref="F22:K22"/>
     <mergeCell ref="B118:D118"/>
     <mergeCell ref="F51:G51"/>
     <mergeCell ref="D62:F62"/>
@@ -5415,7 +5113,6 @@
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="H51:K51"/>
     <mergeCell ref="B65:C65"/>
-    <mergeCell ref="F18"/>
     <mergeCell ref="F52:G52"/>
     <mergeCell ref="D63:F63"/>
     <mergeCell ref="E117:G117"/>
@@ -5423,7 +5120,6 @@
     <mergeCell ref="E76:I76"/>
     <mergeCell ref="D30:K30"/>
     <mergeCell ref="D82:E82"/>
-    <mergeCell ref="F17"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="B44:K44"/>
     <mergeCell ref="G94:K94"/>
@@ -5432,8 +5128,7 @@
     <mergeCell ref="D29:K29"/>
     <mergeCell ref="B52:D52"/>
     <mergeCell ref="E75:I75"/>
-    <mergeCell ref="F22"/>
-    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F21:K21"/>
     <mergeCell ref="F88:J88"/>
   </mergeCells>
   <conditionalFormatting sqref="B4">
@@ -5523,163 +5218,100 @@
       <formula>Calc!$B$57="Critical"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F18">
-    <cfRule type="dataBar" priority="26">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F19">
-    <cfRule type="dataBar" priority="27">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F20">
-    <cfRule type="dataBar" priority="28">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F21">
-    <cfRule type="dataBar" priority="29">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F22">
-    <cfRule type="dataBar" priority="30">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
-    <cfRule type="dataBar" priority="31">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F24">
-    <cfRule type="dataBar" priority="32">
-      <dataBar showValue="0">
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="004F2D7F"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E18:E24">
-    <cfRule type="cellIs" priority="33" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="26" operator="equal" dxfId="6">
       <formula>"Partial"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="34" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="1">
       <formula>"Informed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="35" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="28" operator="equal" dxfId="0">
       <formula>"Repeatable"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="36" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="29" operator="equal" dxfId="4">
       <formula>"Adaptive"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H38:H41">
-    <cfRule type="cellIs" priority="37" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="30" operator="equal" dxfId="0">
       <formula>"Low"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="31" operator="equal" dxfId="1">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="39" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="32" operator="equal" dxfId="2">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="40" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="33" operator="equal" dxfId="3">
       <formula>"Very high"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F46:F53">
-    <cfRule type="cellIs" priority="41" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="34" operator="equal" dxfId="0">
       <formula>"Well addressed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="35" operator="equal" dxfId="1">
       <formula>"Partially addressed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="43" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="36" operator="equal" dxfId="2">
       <formula>"Needs attention"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D57:D67">
-    <cfRule type="expression" priority="44" dxfId="3">
+    <cfRule type="expression" priority="37" dxfId="3">
       <formula>ISNUMBER(SEARCH("Not met",LEFT($D57,25)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="45" dxfId="2">
+    <cfRule type="expression" priority="38" dxfId="2">
       <formula>ISNUMBER(SEARCH("Minimal",LEFT($D57,25)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="46" dxfId="1">
+    <cfRule type="expression" priority="39" dxfId="1">
       <formula>ISNUMBER(SEARCH("Partially",LEFT($D57,25)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="47" dxfId="0">
+    <cfRule type="expression" priority="40" dxfId="0">
       <formula>ISNUMBER(SEARCH("Largely",LEFT($D57,25)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="48" dxfId="4">
+    <cfRule type="expression" priority="41" dxfId="4">
       <formula>ISNUMBER(SEARCH("Fully",LEFT($D57,25)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B80:B90">
-    <cfRule type="expression" priority="49" dxfId="2">
+    <cfRule type="expression" priority="42" dxfId="2">
       <formula>LEFT($B80,9)="Immediate"</formula>
     </cfRule>
-    <cfRule type="expression" priority="50" dxfId="1">
+    <cfRule type="expression" priority="43" dxfId="1">
       <formula>LEFT($B80,5)="Short"</formula>
     </cfRule>
-    <cfRule type="expression" priority="51" dxfId="0">
+    <cfRule type="expression" priority="44" dxfId="0">
       <formula>LEFT($B80,6)="Medium"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F95:F102">
-    <cfRule type="cellIs" priority="52" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="45" operator="equal" dxfId="0">
       <formula>"On track"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="53" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="46" operator="equal" dxfId="1">
       <formula>"Partial gap"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="54" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="47" operator="equal" dxfId="2">
       <formula>"Significant gap"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E95:E102">
-    <cfRule type="cellIs" priority="55" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="48" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E106:E110">
-    <cfRule type="cellIs" priority="56" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="49" operator="equal" dxfId="2">
       <formula>"Priority"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="50" operator="equal" dxfId="1">
       <formula>"Advised"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="58" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="51" operator="equal" dxfId="0">
       <formula>"Optional"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="52" operator="equal" dxfId="4">
       <formula>"Sustain"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5699,7 +5331,6 @@
     <brk id="68" min="0" max="16383" man="1"/>
     <brk id="91" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Readiness tool: domains now AI Governance, AI Risk & Security, Training & Awareness, Strategy & Value, Data & Technology
- Protect AI + AI Threats + AI risk-management questions combined into AI Risk & Security
- Questions regrouped by domain; sample responses, questionnaire and sample report regenerated
- Report: chart spacing, page numbers start at 1, headers kept with their rows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
@@ -2089,11 +2089,671 @@
       </c>
       <c r="C15" s="31" t="inlineStr">
         <is>
+          <t>AI Governance
+AI governance structure &amp; accountability</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Is there a defined AI governance structure - board / executive oversight, an AI committee with decision rights, named owners for every AI system and clear three-lines-of-defence responsibilities?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: board / ExCo terms of reference covering AI, AI committee charter, RACI, AI system owner register, internal-audit coverage.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E15" s="33" t="n"/>
+      <c r="F15" s="37" t="str">
+        <f>IF(L15="","",INDEX(QBank!$C$22:$C$26,L15))</f>
+        <v/>
+      </c>
+      <c r="G15" s="35" t="str">
+        <f>IF(L15="","Not answered",INDEX(QBank!$D$22:$D$26,L15))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H15" s="36" t="str">
+        <f>IF(L15="","",INDEX(QBank!$E$22:$E$26,L15))</f>
+        <v/>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>GL-1, GL-2, GL-7, AA-1</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Mandatory Requirement</t>
+        </is>
+      </c>
+      <c r="L15" t="str">
+        <f>IF(E15="","",IFERROR(MATCH(E15,QBank!$B$22:$B$26,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="96" customHeight="1">
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>AI Governance
+AI policy, acceptable use &amp; regulatory compliance</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Do you have an approved AI (acceptable-use) policy and a process to identify and comply with applicable AI-related regulation (e.g., Bahrain PDPL, CBB rules, EU AI Act)?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI policy, approved-tools list, staff acknowledgements, obligations register, compliance reviews.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E16" s="33" t="n"/>
+      <c r="F16" s="37" t="str">
+        <f>IF(L16="","",INDEX(QBank!$C$27:$C$31,L16))</f>
+        <v/>
+      </c>
+      <c r="G16" s="35" t="str">
+        <f>IF(L16="","Not answered",INDEX(QBank!$D$27:$D$31,L16))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H16" s="36" t="str">
+        <f>IF(L16="","",INDEX(QBank!$E$27:$E$31,L16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>GL-5, RO-1, RO-5</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>⟳ Compliance Obligation</t>
+        </is>
+      </c>
+      <c r="L16" t="str">
+        <f>IF(E16="","",IFERROR(MATCH(E16,QBank!$B$27:$B$31,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>AI Governance
+Responsible-AI guardrails &amp; human oversight</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Are there practical guardrails for fairness, transparency and human oversight, overseen by an AI committee or centre of excellence?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: committee / CoE charter, guardrail standards, human-in-charge procedures, bias tests, AI disclosures, appeal routes.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E17" s="33" t="n"/>
+      <c r="F17" s="37" t="str">
+        <f>IF(L17="","",INDEX(QBank!$C$32:$C$36,L17))</f>
+        <v/>
+      </c>
+      <c r="G17" s="35" t="str">
+        <f>IF(L17="","Not answered",INDEX(QBank!$D$32:$D$36,L17))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H17" s="36" t="str">
+        <f>IF(L17="","",INDEX(QBank!$E$32:$E$36,L17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>⚖ Ethical Consideration</t>
+        </is>
+      </c>
+      <c r="L17" t="str">
+        <f>IF(E17="","",IFERROR(MATCH(E17,QBank!$B$32:$B$36,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="96" customHeight="1">
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>AI Governance
+AI incidents, monitoring &amp; assurance</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Are AI incidents detected, managed and reported, and is AI governance subject to internal audit or independent assurance?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI incident categories, notification criteria, incident logs, internal-audit reports, vendor assurance, certification status.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="37" t="str">
+        <f>IF(L18="","",INDEX(QBank!$C$37:$C$41,L18))</f>
+        <v/>
+      </c>
+      <c r="G18" s="35" t="str">
+        <f>IF(L18="","Not answered",INDEX(QBank!$D$37:$D$41,L18))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H18" s="36" t="str">
+        <f>IF(L18="","",INDEX(QBank!$E$37:$E$41,L18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>⟳ Compliance Obligation</t>
+        </is>
+      </c>
+      <c r="L18" t="str">
+        <f>IF(E18="","",IFERROR(MATCH(E18,QBank!$B$37:$B$41,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="96" customHeight="1">
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+AI risk management framework</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Is there a documented AI risk management framework - risk taxonomy, assessment method, scoring scales and treatment process - integrated with enterprise risk management?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI risk framework / methodology (e.g., aligned to ISO/IEC 23894 or NIST AI RMF), AI risk register, link to the enterprise risk register, completed assessments.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E19" s="33" t="n"/>
+      <c r="F19" s="37" t="str">
+        <f>IF(L19="","",INDEX(QBank!$C$42:$C$46,L19))</f>
+        <v/>
+      </c>
+      <c r="G19" s="35" t="str">
+        <f>IF(L19="","Not answered",INDEX(QBank!$D$42:$D$46,L19))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H19" s="36" t="str">
+        <f>IF(L19="","",INDEX(QBank!$E$42:$E$46,L19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>RM-1, RM-2, RM-3, RM-5</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Mandatory Requirement</t>
+        </is>
+      </c>
+      <c r="L19" t="str">
+        <f>IF(E19="","",IFERROR(MATCH(E19,QBank!$B$42:$B$46,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+AI risk appetite, KRIs &amp; reporting</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Has the board approved an AI risk appetite with measurable tolerances, and are key risk indicators (KRIs) monitored and reported with defined escalation?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: approved AI risk appetite statement, KRI library with thresholds, risk dashboards, escalation and breach records.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="37" t="str">
+        <f>IF(L20="","",INDEX(QBank!$C$47:$C$51,L20))</f>
+        <v/>
+      </c>
+      <c r="G20" s="35" t="str">
+        <f>IF(L20="","Not answered",INDEX(QBank!$D$47:$D$51,L20))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H20" s="36" t="str">
+        <f>IF(L20="","",INDEX(QBank!$E$47:$E$51,L20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>RM-6, RM-4, GL-1</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Mandatory Requirement</t>
+        </is>
+      </c>
+      <c r="L20" t="str">
+        <f>IF(E20="","",IFERROR(MATCH(E20,QBank!$B$47:$B$51,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+AI inventory &amp; risk / impact assessment</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Do you maintain an inventory of AI systems with named owners, and assess AI risks and impacts (including third-party AI) before and after deployment?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI register, risk-tiering records, impact assessments, vendor AI due diligence, re-assessment records.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E21" s="33" t="n"/>
+      <c r="F21" s="37" t="str">
+        <f>IF(L21="","",INDEX(QBank!$C$52:$C$56,L21))</f>
+        <v/>
+      </c>
+      <c r="G21" s="35" t="str">
+        <f>IF(L21="","Not answered",INDEX(QBank!$D$52:$D$56,L21))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H21" s="36" t="str">
+        <f>IF(L21="","",INDEX(QBank!$E$52:$E$56,L21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>GL-8, RM-2, RM-5, TP-2</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Mandatory Requirement</t>
+        </is>
+      </c>
+      <c r="L21" t="str">
+        <f>IF(E21="","",IFERROR(MATCH(E21,QBank!$B$52:$B$56,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+Third-party &amp; AI supply-chain risk</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Are AI vendors, AI features in purchased software and foundation-model providers risk-assessed before use, with AI-specific contract clauses and ongoing monitoring?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI vendor due-diligence questionnaire, contract clauses (no training on your data, residency, incident notice, audit rights), vendor assurance (ISO/IEC 42001, SOC 2), review records.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="37" t="str">
+        <f>IF(L22="","",INDEX(QBank!$C$57:$C$61,L22))</f>
+        <v/>
+      </c>
+      <c r="G22" s="35" t="str">
+        <f>IF(L22="","Not answered",INDEX(QBank!$D$57:$D$61,L22))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H22" s="36" t="str">
+        <f>IF(L22="","",INDEX(QBank!$E$57:$E$61,L22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>TP-1, TP-2, TP-3, SE-7, LC-6</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>⟳ Compliance Obligation</t>
+        </is>
+      </c>
+      <c r="L22" t="str">
+        <f>IF(E22="","",IFERROR(MATCH(E22,QBank!$B$57:$B$61,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+Securing AI systems</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Are AI systems protected with least-privilege access, secure development and testing (incl. red teaming for prompt injection), and runtime logging?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI threat models, access reviews (incl. agent identities), AI red-team reports, guardrail and sandbox configurations, audit logs. Detailed test: GT AI Security &amp; Agent Audit Checklist.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="37" t="str">
+        <f>IF(L23="","",INDEX(QBank!$C$62:$C$66,L23))</f>
+        <v/>
+      </c>
+      <c r="G23" s="35" t="str">
+        <f>IF(L23="","Not answered",INDEX(QBank!$D$62:$D$66,L23))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H23" s="36" t="str">
+        <f>IF(L23="","",INDEX(QBank!$E$62:$E$66,L23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>⚠ Mandatory Requirement</t>
+        </is>
+      </c>
+      <c r="L23" t="str">
+        <f>IF(E23="","",IFERROR(MATCH(E23,QBank!$B$62:$B$66,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="96" customHeight="1">
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>AI Risk &amp; Security
+Defending against AI-enabled threats</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Is the organisation prepared for AI-enabled attacks such as deepfake impersonation, AI-crafted phishing and automated exploitation?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: AI threat intelligence, out-of-band verification procedures, deepfake simulations, SOC use cases, playbooks, patch metrics.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="37" t="str">
+        <f>IF(L24="","",INDEX(QBank!$C$67:$C$71,L24))</f>
+        <v/>
+      </c>
+      <c r="G24" s="35" t="str">
+        <f>IF(L24="","Not answered",INDEX(QBank!$D$67:$D$71,L24))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H24" s="36" t="str">
+        <f>IF(L24="","",INDEX(QBank!$E$67:$E$71,L24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>AT-1, AT-2, AT-3, AT-4</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>☆ Recommended</t>
+        </is>
+      </c>
+      <c r="L24" t="str">
+        <f>IF(E24="","",IFERROR(MATCH(E24,QBank!$B$67:$B$71,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="96" customHeight="1">
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>Training &amp; Awareness
+AI training, literacy &amp; awareness</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Have staff received AI literacy training appropriate to their role, and are specialist AI, governance and security skills being developed?</t>
+          </r>
+          <r>
+            <rPr>
+              <i val="1"/>
+              <color rgb="006B6B6B"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve">
+Evidence: training curricula, completion records, role-based pathways, deepfake / phishing simulations, workforce plan.</t>
+          </r>
+        </is>
+      </c>
+      <c r="E25" s="33" t="n"/>
+      <c r="F25" s="37" t="str">
+        <f>IF(L25="","",INDEX(QBank!$C$72:$C$76,L25))</f>
+        <v/>
+      </c>
+      <c r="G25" s="35" t="str">
+        <f>IF(L25="","Not answered",INDEX(QBank!$D$72:$D$76,L25))</f>
+        <v>Not answered</v>
+      </c>
+      <c r="H25" s="36" t="str">
+        <f>IF(L25="","",INDEX(QBank!$E$72:$E$76,L25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>GL-4, RS-9</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>⟳ Compliance Obligation</t>
+        </is>
+      </c>
+      <c r="L25" t="str">
+        <f>IF(E25="","",IFERROR(MATCH(E25,QBank!$B$72:$B$76,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
           <t>Strategy &amp; Value
 AI strategy &amp; executive ownership</t>
         </is>
       </c>
-      <c r="D15" s="32" t="inlineStr">
+      <c r="D26" s="32" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2113,47 +2773,47 @@
           </r>
         </is>
       </c>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="37" t="str">
-        <f>IF(L15="","",INDEX(QBank!$C$22:$C$26,L15))</f>
-        <v/>
-      </c>
-      <c r="G15" s="35" t="str">
-        <f>IF(L15="","Not answered",INDEX(QBank!$D$22:$D$26,L15))</f>
+      <c r="E26" s="33" t="n"/>
+      <c r="F26" s="37" t="str">
+        <f>IF(L26="","",INDEX(QBank!$C$77:$C$81,L26))</f>
+        <v/>
+      </c>
+      <c r="G26" s="35" t="str">
+        <f>IF(L26="","Not answered",INDEX(QBank!$D$77:$D$81,L26))</f>
         <v>Not answered</v>
       </c>
-      <c r="H15" s="36" t="str">
-        <f>IF(L15="","",INDEX(QBank!$E$22:$E$26,L15))</f>
-        <v/>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="H26" s="36" t="str">
+        <f>IF(L26="","",INDEX(QBank!$E$77:$E$81,L26))</f>
+        <v/>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>GL-1, GL-3</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J26" s="7" t="inlineStr">
         <is>
           <t>☆ Recommended</t>
         </is>
       </c>
-      <c r="L15" t="str">
-        <f>IF(E15="","",IFERROR(MATCH(E15,QBank!$B$22:$B$26,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="96" customHeight="1">
-      <c r="B16" s="30" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="L26" t="str">
+        <f>IF(E26="","",IFERROR(MATCH(E26,QBank!$B$77:$B$81,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="96" customHeight="1">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>Strategy &amp; Value
 Use-case portfolio &amp; value realisation</t>
         </is>
       </c>
-      <c r="D16" s="32" t="inlineStr">
+      <c r="D27" s="32" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2173,587 +2833,47 @@
           </r>
         </is>
       </c>
-      <c r="E16" s="33" t="n"/>
-      <c r="F16" s="37" t="str">
-        <f>IF(L16="","",INDEX(QBank!$C$27:$C$31,L16))</f>
-        <v/>
-      </c>
-      <c r="G16" s="35" t="str">
-        <f>IF(L16="","Not answered",INDEX(QBank!$D$27:$D$31,L16))</f>
+      <c r="E27" s="33" t="n"/>
+      <c r="F27" s="37" t="str">
+        <f>IF(L27="","",INDEX(QBank!$C$82:$C$86,L27))</f>
+        <v/>
+      </c>
+      <c r="G27" s="35" t="str">
+        <f>IF(L27="","Not answered",INDEX(QBank!$D$82:$D$86,L27))</f>
         <v>Not answered</v>
       </c>
-      <c r="H16" s="36" t="str">
-        <f>IF(L16="","",INDEX(QBank!$E$27:$E$31,L16))</f>
-        <v/>
-      </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="H27" s="36" t="str">
+        <f>IF(L27="","",INDEX(QBank!$E$82:$E$86,L27))</f>
+        <v/>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
         <is>
           <t>GL-6, GL-5</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>☆ Recommended</t>
         </is>
       </c>
-      <c r="L16" t="str">
-        <f>IF(E16="","",IFERROR(MATCH(E16,QBank!$B$27:$B$31,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="96" customHeight="1">
-      <c r="B17" s="30" t="inlineStr">
-        <is>
-          <t>Q7</t>
-        </is>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI governance structure &amp; accountability</t>
-        </is>
-      </c>
-      <c r="D17" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is there a defined AI governance structure - board / executive oversight, an AI committee with decision rights, named owners for every AI system and clear three-lines-of-defence responsibilities?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: board / ExCo terms of reference covering AI, AI committee charter, RACI, AI system owner register, internal-audit coverage.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E17" s="33" t="n"/>
-      <c r="F17" s="37" t="str">
-        <f>IF(L17="","",INDEX(QBank!$C$32:$C$36,L17))</f>
-        <v/>
-      </c>
-      <c r="G17" s="35" t="str">
-        <f>IF(L17="","Not answered",INDEX(QBank!$D$32:$D$36,L17))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H17" s="36" t="str">
-        <f>IF(L17="","",INDEX(QBank!$E$32:$E$36,L17))</f>
-        <v/>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>GL-1, GL-2, GL-7, AA-1</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Mandatory Requirement</t>
-        </is>
-      </c>
-      <c r="L17" t="str">
-        <f>IF(E17="","",IFERROR(MATCH(E17,QBank!$B$32:$B$36,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="96" customHeight="1">
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>Q8</t>
-        </is>
-      </c>
-      <c r="C18" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI policy, acceptable use &amp; regulatory compliance</t>
-        </is>
-      </c>
-      <c r="D18" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Do you have an approved AI (acceptable-use) policy and a process to identify and comply with applicable AI-related regulation (e.g., Bahrain PDPL, CBB rules, EU AI Act)?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI policy, approved-tools list, staff acknowledgements, obligations register, compliance reviews.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E18" s="33" t="n"/>
-      <c r="F18" s="37" t="str">
-        <f>IF(L18="","",INDEX(QBank!$C$37:$C$41,L18))</f>
-        <v/>
-      </c>
-      <c r="G18" s="35" t="str">
-        <f>IF(L18="","Not answered",INDEX(QBank!$D$37:$D$41,L18))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H18" s="36" t="str">
-        <f>IF(L18="","",INDEX(QBank!$E$37:$E$41,L18))</f>
-        <v/>
-      </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>GL-5, RO-1, RO-5</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>⟳ Compliance Obligation</t>
-        </is>
-      </c>
-      <c r="L18" t="str">
-        <f>IF(E18="","",IFERROR(MATCH(E18,QBank!$B$37:$B$41,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="96" customHeight="1">
-      <c r="B19" s="30" t="inlineStr">
-        <is>
-          <t>Q9</t>
-        </is>
-      </c>
-      <c r="C19" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI risk management framework</t>
-        </is>
-      </c>
-      <c r="D19" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is there a documented AI risk management framework - risk taxonomy, assessment method, scoring scales and treatment process - integrated with enterprise risk management?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI risk framework / methodology (e.g., aligned to ISO/IEC 23894 or NIST AI RMF), AI risk register, link to the enterprise risk register, completed assessments.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E19" s="33" t="n"/>
-      <c r="F19" s="37" t="str">
-        <f>IF(L19="","",INDEX(QBank!$C$42:$C$46,L19))</f>
-        <v/>
-      </c>
-      <c r="G19" s="35" t="str">
-        <f>IF(L19="","Not answered",INDEX(QBank!$D$42:$D$46,L19))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H19" s="36" t="str">
-        <f>IF(L19="","",INDEX(QBank!$E$42:$E$46,L19))</f>
-        <v/>
-      </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>RM-1, RM-2, RM-3, RM-5</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Mandatory Requirement</t>
-        </is>
-      </c>
-      <c r="L19" t="str">
-        <f>IF(E19="","",IFERROR(MATCH(E19,QBank!$B$42:$B$46,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="96" customHeight="1">
-      <c r="B20" s="30" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="C20" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI risk appetite, KRIs &amp; reporting</t>
-        </is>
-      </c>
-      <c r="D20" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Has the board approved an AI risk appetite with measurable tolerances, and are key risk indicators (KRIs) monitored and reported with defined escalation?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: approved AI risk appetite statement, KRI library with thresholds, risk dashboards, escalation and breach records.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E20" s="33" t="n"/>
-      <c r="F20" s="37" t="str">
-        <f>IF(L20="","",INDEX(QBank!$C$47:$C$51,L20))</f>
-        <v/>
-      </c>
-      <c r="G20" s="35" t="str">
-        <f>IF(L20="","Not answered",INDEX(QBank!$D$47:$D$51,L20))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H20" s="36" t="str">
-        <f>IF(L20="","",INDEX(QBank!$E$47:$E$51,L20))</f>
-        <v/>
-      </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>RM-6, RM-4, GL-1</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Mandatory Requirement</t>
-        </is>
-      </c>
-      <c r="L20" t="str">
-        <f>IF(E20="","",IFERROR(MATCH(E20,QBank!$B$47:$B$51,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="96" customHeight="1">
-      <c r="B21" s="30" t="inlineStr">
-        <is>
-          <t>Q11</t>
-        </is>
-      </c>
-      <c r="C21" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI inventory &amp; risk / impact assessment</t>
-        </is>
-      </c>
-      <c r="D21" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Do you maintain an inventory of AI systems with named owners, and assess AI risks and impacts (including third-party AI) before and after deployment?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI register, risk-tiering records, impact assessments, vendor AI due diligence, re-assessment records.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E21" s="33" t="n"/>
-      <c r="F21" s="37" t="str">
-        <f>IF(L21="","",INDEX(QBank!$C$52:$C$56,L21))</f>
-        <v/>
-      </c>
-      <c r="G21" s="35" t="str">
-        <f>IF(L21="","Not answered",INDEX(QBank!$D$52:$D$56,L21))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H21" s="36" t="str">
-        <f>IF(L21="","",INDEX(QBank!$E$52:$E$56,L21))</f>
-        <v/>
-      </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>GL-8, RM-2, RM-5, TP-2</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Mandatory Requirement</t>
-        </is>
-      </c>
-      <c r="L21" t="str">
-        <f>IF(E21="","",IFERROR(MATCH(E21,QBank!$B$52:$B$56,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="96" customHeight="1">
-      <c r="B22" s="30" t="inlineStr">
-        <is>
-          <t>Q12</t>
-        </is>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-Third-party &amp; AI supply-chain risk</t>
-        </is>
-      </c>
-      <c r="D22" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are AI vendors, AI features in purchased software and foundation-model providers risk-assessed before use, with AI-specific contract clauses and ongoing monitoring?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI vendor due-diligence questionnaire, contract clauses (no training on your data, residency, incident notice, audit rights), vendor assurance (ISO/IEC 42001, SOC 2), review records.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E22" s="33" t="n"/>
-      <c r="F22" s="37" t="str">
-        <f>IF(L22="","",INDEX(QBank!$C$57:$C$61,L22))</f>
-        <v/>
-      </c>
-      <c r="G22" s="35" t="str">
-        <f>IF(L22="","Not answered",INDEX(QBank!$D$57:$D$61,L22))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H22" s="36" t="str">
-        <f>IF(L22="","",INDEX(QBank!$E$57:$E$61,L22))</f>
-        <v/>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>TP-1, TP-2, TP-3, SE-7, LC-6</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>⟳ Compliance Obligation</t>
-        </is>
-      </c>
-      <c r="L22" t="str">
-        <f>IF(E22="","",IFERROR(MATCH(E22,QBank!$B$57:$B$61,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="96" customHeight="1">
-      <c r="B23" s="30" t="inlineStr">
-        <is>
-          <t>Q13</t>
-        </is>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-Responsible-AI guardrails &amp; human oversight</t>
-        </is>
-      </c>
-      <c r="D23" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are there practical guardrails for fairness, transparency and human oversight, overseen by an AI committee or centre of excellence?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: committee / CoE charter, guardrail standards, human-in-charge procedures, bias tests, AI disclosures, appeal routes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E23" s="33" t="n"/>
-      <c r="F23" s="37" t="str">
-        <f>IF(L23="","",INDEX(QBank!$C$62:$C$66,L23))</f>
-        <v/>
-      </c>
-      <c r="G23" s="35" t="str">
-        <f>IF(L23="","Not answered",INDEX(QBank!$D$62:$D$66,L23))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H23" s="36" t="str">
-        <f>IF(L23="","",INDEX(QBank!$E$62:$E$66,L23))</f>
-        <v/>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>⚖ Ethical Consideration</t>
-        </is>
-      </c>
-      <c r="L23" t="str">
-        <f>IF(E23="","",IFERROR(MATCH(E23,QBank!$B$62:$B$66,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="96" customHeight="1">
-      <c r="B24" s="30" t="inlineStr">
-        <is>
-          <t>Q14</t>
-        </is>
-      </c>
-      <c r="C24" s="31" t="inlineStr">
-        <is>
-          <t>Governance, Risk &amp; Compliance
-AI incidents, monitoring &amp; assurance</t>
-        </is>
-      </c>
-      <c r="D24" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are AI incidents detected, managed and reported, and is AI governance subject to internal audit or independent assurance?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI incident categories, notification criteria, incident logs, internal-audit reports, vendor assurance, certification status.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E24" s="33" t="n"/>
-      <c r="F24" s="37" t="str">
-        <f>IF(L24="","",INDEX(QBank!$C$67:$C$71,L24))</f>
-        <v/>
-      </c>
-      <c r="G24" s="35" t="str">
-        <f>IF(L24="","Not answered",INDEX(QBank!$D$67:$D$71,L24))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H24" s="36" t="str">
-        <f>IF(L24="","",INDEX(QBank!$E$67:$E$71,L24))</f>
-        <v/>
-      </c>
-      <c r="I24" s="7" t="inlineStr">
-        <is>
-          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
-        </is>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>⟳ Compliance Obligation</t>
-        </is>
-      </c>
-      <c r="L24" t="str">
-        <f>IF(E24="","",IFERROR(MATCH(E24,QBank!$B$67:$B$71,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="96" customHeight="1">
-      <c r="B25" s="30" t="inlineStr">
-        <is>
-          <t>Q15</t>
-        </is>
-      </c>
-      <c r="C25" s="31" t="inlineStr">
-        <is>
-          <t>People &amp; Skills
-AI literacy &amp; capability</t>
-        </is>
-      </c>
-      <c r="D25" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Have staff received AI literacy training appropriate to their role, and are specialist AI, governance and security skills being developed?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: training curricula, completion records, role-based pathways, deepfake / phishing simulations, workforce plan.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E25" s="33" t="n"/>
-      <c r="F25" s="37" t="str">
-        <f>IF(L25="","",INDEX(QBank!$C$72:$C$76,L25))</f>
-        <v/>
-      </c>
-      <c r="G25" s="35" t="str">
-        <f>IF(L25="","Not answered",INDEX(QBank!$D$72:$D$76,L25))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H25" s="36" t="str">
-        <f>IF(L25="","",INDEX(QBank!$E$72:$E$76,L25))</f>
-        <v/>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>GL-4, RS-9</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>⟳ Compliance Obligation</t>
-        </is>
-      </c>
-      <c r="L25" t="str">
-        <f>IF(E25="","",IFERROR(MATCH(E25,QBank!$B$72:$B$76,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="96" customHeight="1">
-      <c r="B26" s="30" t="inlineStr">
-        <is>
-          <t>Q16</t>
-        </is>
-      </c>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="L27" t="str">
+        <f>IF(E27="","",IFERROR(MATCH(E27,QBank!$B$82:$B$86,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="96" customHeight="1">
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
         <is>
           <t>Data &amp; Technology
 Data governance, quality &amp; privacy for AI</t>
         </is>
       </c>
-      <c r="D26" s="32" t="inlineStr">
+      <c r="D28" s="32" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2773,47 +2893,47 @@
           </r>
         </is>
       </c>
-      <c r="E26" s="33" t="n"/>
-      <c r="F26" s="37" t="str">
-        <f>IF(L26="","",INDEX(QBank!$C$77:$C$81,L26))</f>
-        <v/>
-      </c>
-      <c r="G26" s="35" t="str">
-        <f>IF(L26="","Not answered",INDEX(QBank!$D$77:$D$81,L26))</f>
+      <c r="E28" s="33" t="n"/>
+      <c r="F28" s="37" t="str">
+        <f>IF(L28="","",INDEX(QBank!$C$87:$C$91,L28))</f>
+        <v/>
+      </c>
+      <c r="G28" s="35" t="str">
+        <f>IF(L28="","Not answered",INDEX(QBank!$D$87:$D$91,L28))</f>
         <v>Not answered</v>
       </c>
-      <c r="H26" s="36" t="str">
-        <f>IF(L26="","",INDEX(QBank!$E$77:$E$81,L26))</f>
-        <v/>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="H28" s="36" t="str">
+        <f>IF(L28="","",INDEX(QBank!$E$87:$E$91,L28))</f>
+        <v/>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
         <is>
           <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
         </is>
       </c>
-      <c r="J26" s="7" t="inlineStr">
+      <c r="J28" s="7" t="inlineStr">
         <is>
           <t>⟳ Compliance Obligation</t>
         </is>
       </c>
-      <c r="L26" t="str">
-        <f>IF(E26="","",IFERROR(MATCH(E26,QBank!$B$77:$B$81,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="96" customHeight="1">
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t>Q17</t>
-        </is>
-      </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="L28" t="str">
+        <f>IF(E28="","",IFERROR(MATCH(E28,QBank!$B$87:$B$91,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="96" customHeight="1">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
         <is>
           <t>Data &amp; Technology
 AI architecture, integration &amp; monitoring</t>
         </is>
       </c>
-      <c r="D27" s="32" t="inlineStr">
+      <c r="D29" s="32" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2833,47 +2953,47 @@
           </r>
         </is>
       </c>
-      <c r="E27" s="33" t="n"/>
-      <c r="F27" s="37" t="str">
-        <f>IF(L27="","",INDEX(QBank!$C$82:$C$86,L27))</f>
-        <v/>
-      </c>
-      <c r="G27" s="35" t="str">
-        <f>IF(L27="","Not answered",INDEX(QBank!$D$82:$D$86,L27))</f>
+      <c r="E29" s="33" t="n"/>
+      <c r="F29" s="37" t="str">
+        <f>IF(L29="","",INDEX(QBank!$C$92:$C$96,L29))</f>
+        <v/>
+      </c>
+      <c r="G29" s="35" t="str">
+        <f>IF(L29="","Not answered",INDEX(QBank!$D$92:$D$96,L29))</f>
         <v>Not answered</v>
       </c>
-      <c r="H27" s="36" t="str">
-        <f>IF(L27="","",INDEX(QBank!$E$82:$E$86,L27))</f>
-        <v/>
-      </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="H29" s="36" t="str">
+        <f>IF(L29="","",INDEX(QBank!$E$92:$E$96,L29))</f>
+        <v/>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>☆ Recommended</t>
         </is>
       </c>
-      <c r="L27" t="str">
-        <f>IF(E27="","",IFERROR(MATCH(E27,QBank!$B$82:$B$86,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="96" customHeight="1">
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t>Q18</t>
-        </is>
-      </c>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="L29" t="str">
+        <f>IF(E29="","",IFERROR(MATCH(E29,QBank!$B$92:$B$96,0),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="96" customHeight="1">
+      <c r="B30" s="30" t="inlineStr">
+        <is>
+          <t>Q20</t>
+        </is>
+      </c>
+      <c r="C30" s="31" t="inlineStr">
         <is>
           <t>Data &amp; Technology
 Model risk management &amp; validation</t>
         </is>
       </c>
-      <c r="D28" s="32" t="inlineStr">
+      <c r="D30" s="32" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2893,126 +3013,6 @@
           </r>
         </is>
       </c>
-      <c r="E28" s="33" t="n"/>
-      <c r="F28" s="37" t="str">
-        <f>IF(L28="","",INDEX(QBank!$C$87:$C$91,L28))</f>
-        <v/>
-      </c>
-      <c r="G28" s="35" t="str">
-        <f>IF(L28="","Not answered",INDEX(QBank!$D$87:$D$91,L28))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H28" s="36" t="str">
-        <f>IF(L28="","",INDEX(QBank!$E$87:$E$91,L28))</f>
-        <v/>
-      </c>
-      <c r="I28" s="7" t="inlineStr">
-        <is>
-          <t>LC-9, RS-6, LC-13, OM-1</t>
-        </is>
-      </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>☆ Recommended</t>
-        </is>
-      </c>
-      <c r="L28" t="str">
-        <f>IF(E28="","",IFERROR(MATCH(E28,QBank!$B$87:$B$91,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="96" customHeight="1">
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t>Q19</t>
-        </is>
-      </c>
-      <c r="C29" s="31" t="inlineStr">
-        <is>
-          <t>AI Security &amp; Threat Risk
-Securing AI systems</t>
-        </is>
-      </c>
-      <c r="D29" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Are AI systems protected with least-privilege access, secure development and testing (incl. red teaming for prompt injection), and runtime logging?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI threat models, access reviews (incl. agent identities), AI red-team reports, guardrail and sandbox configurations, audit logs. Detailed test: GT AI Security &amp; Agent Audit Checklist.</t>
-          </r>
-        </is>
-      </c>
-      <c r="E29" s="33" t="n"/>
-      <c r="F29" s="37" t="str">
-        <f>IF(L29="","",INDEX(QBank!$C$92:$C$96,L29))</f>
-        <v/>
-      </c>
-      <c r="G29" s="35" t="str">
-        <f>IF(L29="","Not answered",INDEX(QBank!$D$92:$D$96,L29))</f>
-        <v>Not answered</v>
-      </c>
-      <c r="H29" s="36" t="str">
-        <f>IF(L29="","",INDEX(QBank!$E$92:$E$96,L29))</f>
-        <v/>
-      </c>
-      <c r="I29" s="7" t="inlineStr">
-        <is>
-          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
-        </is>
-      </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>⚠ Mandatory Requirement</t>
-        </is>
-      </c>
-      <c r="L29" t="str">
-        <f>IF(E29="","",IFERROR(MATCH(E29,QBank!$B$92:$B$96,0),""))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="96" customHeight="1">
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>Q20</t>
-        </is>
-      </c>
-      <c r="C30" s="31" t="inlineStr">
-        <is>
-          <t>AI Security &amp; Threat Risk
-Defending against AI-enabled threats</t>
-        </is>
-      </c>
-      <c r="D30" s="32" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>Is the organisation prepared for AI-enabled attacks such as deepfake impersonation, AI-crafted phishing and automated exploitation?</t>
-          </r>
-          <r>
-            <rPr>
-              <i val="1"/>
-              <color rgb="006B6B6B"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve">
-Evidence: AI threat intelligence, out-of-band verification procedures, deepfake simulations, SOC use cases, playbooks, patch metrics.</t>
-          </r>
-        </is>
-      </c>
       <c r="E30" s="33" t="n"/>
       <c r="F30" s="37" t="str">
         <f>IF(L30="","",INDEX(QBank!$C$97:$C$101,L30))</f>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>AT-1, AT-2, AT-3, AT-4</t>
+          <t>LC-9, RS-6, LC-13, OM-1</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
@@ -3462,7 +3462,7 @@
     <row r="18" ht="25" customHeight="1">
       <c r="B18" s="56" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="C18" s="21" t="n"/>
@@ -3482,7 +3482,7 @@
     <row r="19" ht="25" customHeight="1">
       <c r="B19" s="56" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="C19" s="21" t="n"/>
@@ -3502,7 +3502,7 @@
     <row r="20" ht="25" customHeight="1">
       <c r="B20" s="56" t="inlineStr">
         <is>
-          <t>People &amp; Skills</t>
+          <t>Training &amp; Awareness</t>
         </is>
       </c>
       <c r="C20" s="21" t="n"/>
@@ -3522,7 +3522,7 @@
     <row r="21" ht="25" customHeight="1">
       <c r="B21" s="56" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="C21" s="21" t="n"/>
@@ -3542,7 +3542,7 @@
     <row r="22" ht="25" customHeight="1">
       <c r="B22" s="56" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="C22" s="21" t="n"/>
@@ -3579,7 +3579,7 @@
         <v>Target 70%</v>
       </c>
     </row>
-    <row r="24"/>
+    <row r="24" ht="80" customHeight="1"/>
     <row r="25" ht="26" customHeight="1">
       <c r="B25" s="23" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
     <row r="26" ht="28" customHeight="1">
       <c r="B26" s="61" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="C26" s="21" t="n"/>
@@ -3622,7 +3622,7 @@
     <row r="27" ht="28" customHeight="1">
       <c r="B27" s="61" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="C27" s="21" t="n"/>
@@ -3641,7 +3641,7 @@
     <row r="28" ht="28" customHeight="1">
       <c r="B28" s="61" t="inlineStr">
         <is>
-          <t>People &amp; Skills</t>
+          <t>Training &amp; Awareness</t>
         </is>
       </c>
       <c r="C28" s="21" t="n"/>
@@ -3660,7 +3660,7 @@
     <row r="29" ht="28" customHeight="1">
       <c r="B29" s="61" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="C29" s="21" t="n"/>
@@ -3679,7 +3679,7 @@
     <row r="30" ht="28" customHeight="1">
       <c r="B30" s="61" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="C30" s="21" t="n"/>
@@ -3904,7 +3904,7 @@
       <c r="G42" s="21" t="n"/>
       <c r="H42" s="62" t="str">
         <f>Calc!C76</f>
-        <v>Q13, Q16, Q18</v>
+        <v>Q7, Q18, Q20</v>
       </c>
       <c r="I42" s="21" t="n"/>
       <c r="J42" s="21" t="n"/>
@@ -3929,7 +3929,7 @@
       <c r="G43" s="21" t="n"/>
       <c r="H43" s="62" t="str">
         <f>Calc!C77</f>
-        <v>Q8, Q12, Q16, Q19, Q20</v>
+        <v>Q6, Q12, Q13, Q14, Q18</v>
       </c>
       <c r="I43" s="21" t="n"/>
       <c r="J43" s="21" t="n"/>
@@ -3954,7 +3954,7 @@
       <c r="G44" s="21" t="n"/>
       <c r="H44" s="62" t="str">
         <f>Calc!C78</f>
-        <v>Q13, Q14</v>
+        <v>Q7, Q8</v>
       </c>
       <c r="I44" s="21" t="n"/>
       <c r="J44" s="21" t="n"/>
@@ -3979,7 +3979,7 @@
       <c r="G45" s="21" t="n"/>
       <c r="H45" s="62" t="str">
         <f>Calc!C79</f>
-        <v>Q5, Q7, Q8, Q9, Q10, Q11, Q12, Q14</v>
+        <v>Q5, Q6, Q8, Q9, Q10, Q11, Q12, Q16</v>
       </c>
       <c r="I45" s="21" t="n"/>
       <c r="J45" s="21" t="n"/>
@@ -4004,7 +4004,7 @@
       <c r="G46" s="21" t="n"/>
       <c r="H46" s="62" t="str">
         <f>Calc!C80</f>
-        <v>Q6, Q11</v>
+        <v>Q11, Q17</v>
       </c>
       <c r="I46" s="21" t="n"/>
       <c r="J46" s="21" t="n"/>
@@ -4029,7 +4029,7 @@
       <c r="G47" s="21" t="n"/>
       <c r="H47" s="62" t="str">
         <f>Calc!C81</f>
-        <v>Q13, Q15</v>
+        <v>Q7, Q15</v>
       </c>
       <c r="I47" s="21" t="n"/>
       <c r="J47" s="21" t="n"/>
@@ -4054,7 +4054,7 @@
       <c r="G48" s="21" t="n"/>
       <c r="H48" s="62" t="str">
         <f>Calc!C82</f>
-        <v>Q9, Q14, Q17, Q18, Q19</v>
+        <v>Q8, Q9, Q13, Q19, Q20</v>
       </c>
       <c r="I48" s="21" t="n"/>
       <c r="J48" s="21" t="n"/>
@@ -4079,7 +4079,7 @@
       <c r="G49" s="21" t="n"/>
       <c r="H49" s="62" t="str">
         <f>Calc!C83</f>
-        <v>Q13, Q14</v>
+        <v>Q7, Q8</v>
       </c>
       <c r="I49" s="21" t="n"/>
       <c r="J49" s="21" t="n"/>
@@ -4124,10 +4124,10 @@
     <row r="53" ht="77.5" customHeight="1">
       <c r="B53" s="66" t="inlineStr">
         <is>
-          <t>Q5  AI strategy &amp; executive ownership
-Strategy &amp; Value
-AI Ready7: 1.1
-☆ Recommended</t>
+          <t>Q5  AI governance structure &amp; accountability
+AI Governance
+AI Ready7: 1.1, 2.3
+⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="C53" s="21" t="n"/>
@@ -4138,12 +4138,12 @@
       <c r="E53" s="21" t="n"/>
       <c r="F53" s="21" t="n"/>
       <c r="G53" s="67" t="str">
-        <f>IF('2. Assessment'!F15=1,"N/A - reported as fully met.","Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.")</f>
-        <v>Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.</v>
+        <f>IF('2. Assessment'!F15=1,"N/A - reported as fully met.","Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.")</f>
+        <v>Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.</v>
       </c>
       <c r="H53" s="21" t="n"/>
       <c r="I53" s="67" t="str">
-        <f>IF('2. Assessment'!E15="","",'2. Assessment'!H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-1, GL-3")</f>
+        <f>IF('2. Assessment'!E15="","",'2. Assessment'!H15&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-1, GL-2, GL-7, AA-1")</f>
         <v/>
       </c>
       <c r="J53" s="21" t="n"/>
@@ -4152,10 +4152,10 @@
     <row r="54" ht="77.5" customHeight="1">
       <c r="B54" s="66" t="inlineStr">
         <is>
-          <t>Q6  Use-case portfolio &amp; value realisation
-Strategy &amp; Value
-AI Ready7: 1.2, 1.3
-☆ Recommended</t>
+          <t>Q6  AI policy, acceptable use &amp; regulatory compliance
+AI Governance
+AI Ready7: 2.1, 2.2
+⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="C54" s="21" t="n"/>
@@ -4166,12 +4166,12 @@
       <c r="E54" s="21" t="n"/>
       <c r="F54" s="21" t="n"/>
       <c r="G54" s="67" t="str">
-        <f>IF('2. Assessment'!F16=1,"N/A - reported as fully met.","Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.")</f>
-        <v>Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.</v>
+        <f>IF('2. Assessment'!F16=1,"N/A - reported as fully met.","Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.")</f>
+        <v>Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.</v>
       </c>
       <c r="H54" s="21" t="n"/>
       <c r="I54" s="67" t="str">
-        <f>IF('2. Assessment'!E16="","",'2. Assessment'!H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-6, GL-5")</f>
+        <f>IF('2. Assessment'!E16="","",'2. Assessment'!H16&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-5, RO-1, RO-5")</f>
         <v/>
       </c>
       <c r="J54" s="21" t="n"/>
@@ -4180,10 +4180,10 @@
     <row r="55" ht="77.5" customHeight="1">
       <c r="B55" s="66" t="inlineStr">
         <is>
-          <t>Q7  AI governance structure &amp; accountability
-Governance, Risk &amp; Compliance
-AI Ready7: 1.1, 2.3
-⚠ Mandatory Requirement</t>
+          <t>Q7  Responsible-AI guardrails &amp; human oversight
+AI Governance
+AI Ready7: 2.3, 5.2
+⚖ Ethical Consideration</t>
         </is>
       </c>
       <c r="C55" s="21" t="n"/>
@@ -4194,12 +4194,12 @@
       <c r="E55" s="21" t="n"/>
       <c r="F55" s="21" t="n"/>
       <c r="G55" s="67" t="str">
-        <f>IF('2. Assessment'!F17=1,"N/A - reported as fully met.","Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.")</f>
-        <v>Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.</v>
+        <f>IF('2. Assessment'!F17=1,"N/A - reported as fully met.","Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.")</f>
+        <v>Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.</v>
       </c>
       <c r="H55" s="21" t="n"/>
       <c r="I55" s="67" t="str">
-        <f>IF('2. Assessment'!E17="","",'2. Assessment'!H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-1, GL-2, GL-7, AA-1")</f>
+        <f>IF('2. Assessment'!E17="","",'2. Assessment'!H17&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-7, RS-1, RS-4, RS-5, CO-1, CO-3")</f>
         <v/>
       </c>
       <c r="J55" s="21" t="n"/>
@@ -4208,9 +4208,9 @@
     <row r="56" ht="77.5" customHeight="1">
       <c r="B56" s="66" t="inlineStr">
         <is>
-          <t>Q8  AI policy, acceptable use &amp; regulatory compliance
-Governance, Risk &amp; Compliance
-AI Ready7: 2.1, 2.2
+          <t>Q8  AI incidents, monitoring &amp; assurance
+AI Governance
+AI Ready7: 2.2, 7.4
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4222,12 +4222,12 @@
       <c r="E56" s="21" t="n"/>
       <c r="F56" s="21" t="n"/>
       <c r="G56" s="67" t="str">
-        <f>IF('2. Assessment'!F18=1,"N/A - reported as fully met.","Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.")</f>
-        <v>Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.</v>
+        <f>IF('2. Assessment'!F18=1,"N/A - reported as fully met.","Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.")</f>
+        <v>Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.</v>
       </c>
       <c r="H56" s="21" t="n"/>
       <c r="I56" s="67" t="str">
-        <f>IF('2. Assessment'!E18="","",'2. Assessment'!H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-5, RO-1, RO-5")</f>
+        <f>IF('2. Assessment'!E18="","",'2. Assessment'!H18&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: IM-1, IM-2, IM-3, AA-1, AA-2, RO-4")</f>
         <v/>
       </c>
       <c r="J56" s="21" t="n"/>
@@ -4237,7 +4237,7 @@
       <c r="B57" s="66" t="inlineStr">
         <is>
           <t>Q9  AI risk management framework
-Governance, Risk &amp; Compliance
+AI Risk &amp; Security
 AI Ready7: 2.4
 ⚠ Mandatory Requirement</t>
         </is>
@@ -4265,7 +4265,7 @@
       <c r="B58" s="66" t="inlineStr">
         <is>
           <t>Q10  AI risk appetite, KRIs &amp; reporting
-Governance, Risk &amp; Compliance
+AI Risk &amp; Security
 AI Ready7: 1.1, 4.4
 ⚠ Mandatory Requirement</t>
         </is>
@@ -4293,7 +4293,7 @@
       <c r="B59" s="66" t="inlineStr">
         <is>
           <t>Q11  AI inventory &amp; risk / impact assessment
-Governance, Risk &amp; Compliance
+AI Risk &amp; Security
 AI Ready7: 2.4, 2.5
 ⚠ Mandatory Requirement</t>
         </is>
@@ -4321,7 +4321,7 @@
       <c r="B60" s="66" t="inlineStr">
         <is>
           <t>Q12  Third-party &amp; AI supply-chain risk
-Governance, Risk &amp; Compliance
+AI Risk &amp; Security
 AI Ready7: 2.4, 6.2
 ⟳ Compliance Obligation</t>
         </is>
@@ -4348,10 +4348,10 @@
     <row r="61" ht="77.5" customHeight="1">
       <c r="B61" s="66" t="inlineStr">
         <is>
-          <t>Q13  Responsible-AI guardrails &amp; human oversight
-Governance, Risk &amp; Compliance
-AI Ready7: 2.3, 5.2
-⚖ Ethical Consideration</t>
+          <t>Q13  Securing AI systems
+AI Risk &amp; Security
+AI Ready7: 6.1, 6.2, 6.3, 6.4, 6.5
+⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="C61" s="21" t="n"/>
@@ -4362,12 +4362,12 @@
       <c r="E61" s="21" t="n"/>
       <c r="F61" s="21" t="n"/>
       <c r="G61" s="67" t="str">
-        <f>IF('2. Assessment'!F23=1,"N/A - reported as fully met.","Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.")</f>
-        <v>Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.</v>
+        <f>IF('2. Assessment'!F23=1,"N/A - reported as fully met.","Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.")</f>
+        <v>Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.</v>
       </c>
       <c r="H61" s="21" t="n"/>
       <c r="I61" s="67" t="str">
-        <f>IF('2. Assessment'!E23="","",'2. Assessment'!H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-7, RS-1, RS-4, RS-5, CO-1, CO-3")</f>
+        <f>IF('2. Assessment'!E23="","",'2. Assessment'!H23&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3")</f>
         <v/>
       </c>
       <c r="J61" s="21" t="n"/>
@@ -4376,10 +4376,10 @@
     <row r="62" ht="77.5" customHeight="1">
       <c r="B62" s="66" t="inlineStr">
         <is>
-          <t>Q14  AI incidents, monitoring &amp; assurance
-Governance, Risk &amp; Compliance
-AI Ready7: 2.2, 7.4
-⟳ Compliance Obligation</t>
+          <t>Q14  Defending against AI-enabled threats
+AI Risk &amp; Security
+AI Ready7: 7.1, 7.2, 7.3, 7.4, 7.5
+☆ Recommended</t>
         </is>
       </c>
       <c r="C62" s="21" t="n"/>
@@ -4390,12 +4390,12 @@
       <c r="E62" s="21" t="n"/>
       <c r="F62" s="21" t="n"/>
       <c r="G62" s="67" t="str">
-        <f>IF('2. Assessment'!F24=1,"N/A - reported as fully met.","Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.")</f>
-        <v>Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.</v>
+        <f>IF('2. Assessment'!F24=1,"N/A - reported as fully met.","Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.")</f>
+        <v>Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.</v>
       </c>
       <c r="H62" s="21" t="n"/>
       <c r="I62" s="67" t="str">
-        <f>IF('2. Assessment'!E24="","",'2. Assessment'!H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: IM-1, IM-2, IM-3, AA-1, AA-2, RO-4")</f>
+        <f>IF('2. Assessment'!E24="","",'2. Assessment'!H24&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: AT-1, AT-2, AT-3, AT-4")</f>
         <v/>
       </c>
       <c r="J62" s="21" t="n"/>
@@ -4404,8 +4404,8 @@
     <row r="63" ht="77.5" customHeight="1">
       <c r="B63" s="66" t="inlineStr">
         <is>
-          <t>Q15  AI literacy &amp; capability
-People &amp; Skills
+          <t>Q15  AI training, literacy &amp; awareness
+Training &amp; Awareness
 AI Ready7: 3.1, 3.2, 3.3, 3.4
 ⟳ Compliance Obligation</t>
         </is>
@@ -4432,10 +4432,10 @@
     <row r="64" ht="77.5" customHeight="1">
       <c r="B64" s="66" t="inlineStr">
         <is>
-          <t>Q16  Data governance, quality &amp; privacy for AI
-Data &amp; Technology
-AI Ready7: 5.1, 5.3, 5.4, 5.5
-⟳ Compliance Obligation</t>
+          <t>Q16  AI strategy &amp; executive ownership
+Strategy &amp; Value
+AI Ready7: 1.1
+☆ Recommended</t>
         </is>
       </c>
       <c r="C64" s="21" t="n"/>
@@ -4446,23 +4446,23 @@
       <c r="E64" s="21" t="n"/>
       <c r="F64" s="21" t="n"/>
       <c r="G64" s="67" t="str">
-        <f>IF('2. Assessment'!F26=1,"N/A - reported as fully met.","Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.")</f>
-        <v>Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.</v>
+        <f>IF('2. Assessment'!F26=1,"N/A - reported as fully met.","Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.")</f>
+        <v>Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.</v>
       </c>
       <c r="H64" s="21" t="n"/>
       <c r="I64" s="67" t="str">
-        <f>IF('2. Assessment'!E26="","",'2. Assessment'!H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-1, SE-4, PR-1, PR-4, PR-5, PR-6")</f>
+        <f>IF('2. Assessment'!E26="","",'2. Assessment'!H26&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-1, GL-3")</f>
         <v/>
       </c>
       <c r="J64" s="21" t="n"/>
       <c r="K64" s="21" t="n"/>
     </row>
-    <row r="65" ht="88" customHeight="1">
+    <row r="65" ht="77.5" customHeight="1">
       <c r="B65" s="66" t="inlineStr">
         <is>
-          <t>Q17  AI architecture, integration &amp; monitoring
-Data &amp; Technology
-AI Ready7: 4.1, 4.2, 4.3, 4.4, 4.5
+          <t>Q17  Use-case portfolio &amp; value realisation
+Strategy &amp; Value
+AI Ready7: 1.2, 1.3
 ☆ Recommended</t>
         </is>
       </c>
@@ -4474,12 +4474,12 @@
       <c r="E65" s="21" t="n"/>
       <c r="F65" s="21" t="n"/>
       <c r="G65" s="67" t="str">
-        <f>IF('2. Assessment'!F27=1,"N/A - reported as fully met.","Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.")</f>
-        <v>Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.</v>
+        <f>IF('2. Assessment'!F27=1,"N/A - reported as fully met.","Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.")</f>
+        <v>Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.</v>
       </c>
       <c r="H65" s="21" t="n"/>
       <c r="I65" s="67" t="str">
-        <f>IF('2. Assessment'!E27="","",'2. Assessment'!H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6")</f>
+        <f>IF('2. Assessment'!E27="","",'2. Assessment'!H27&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: GL-6, GL-5")</f>
         <v/>
       </c>
       <c r="J65" s="21" t="n"/>
@@ -4488,10 +4488,10 @@
     <row r="66" ht="77.5" customHeight="1">
       <c r="B66" s="66" t="inlineStr">
         <is>
-          <t>Q18  Model risk management &amp; validation
+          <t>Q18  Data governance, quality &amp; privacy for AI
 Data &amp; Technology
-AI Ready7: 4.4, 6.3
-☆ Recommended</t>
+AI Ready7: 5.1, 5.3, 5.4, 5.5
+⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="C66" s="21" t="n"/>
@@ -4502,24 +4502,24 @@
       <c r="E66" s="21" t="n"/>
       <c r="F66" s="21" t="n"/>
       <c r="G66" s="67" t="str">
-        <f>IF('2. Assessment'!F28=1,"N/A - reported as fully met.","Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.")</f>
-        <v>Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.</v>
+        <f>IF('2. Assessment'!F28=1,"N/A - reported as fully met.","Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.")</f>
+        <v>Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.</v>
       </c>
       <c r="H66" s="21" t="n"/>
       <c r="I66" s="67" t="str">
-        <f>IF('2. Assessment'!E28="","",'2. Assessment'!H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-9, RS-6, LC-13, OM-1")</f>
+        <f>IF('2. Assessment'!E28="","",'2. Assessment'!H28&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-1, SE-4, PR-1, PR-4, PR-5, PR-6")</f>
         <v/>
       </c>
       <c r="J66" s="21" t="n"/>
       <c r="K66" s="21" t="n"/>
     </row>
-    <row r="67" ht="77.5" customHeight="1">
+    <row r="67" ht="88" customHeight="1">
       <c r="B67" s="66" t="inlineStr">
         <is>
-          <t>Q19  Securing AI systems
-AI Security &amp; Threat Risk
-AI Ready7: 6.1, 6.2, 6.3, 6.4, 6.5
-⚠ Mandatory Requirement</t>
+          <t>Q19  AI architecture, integration &amp; monitoring
+Data &amp; Technology
+AI Ready7: 4.1, 4.2, 4.3, 4.4, 4.5
+☆ Recommended</t>
         </is>
       </c>
       <c r="C67" s="21" t="n"/>
@@ -4530,12 +4530,12 @@
       <c r="E67" s="21" t="n"/>
       <c r="F67" s="21" t="n"/>
       <c r="G67" s="67" t="str">
-        <f>IF('2. Assessment'!F29=1,"N/A - reported as fully met.","Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.")</f>
-        <v>Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.</v>
+        <f>IF('2. Assessment'!F29=1,"N/A - reported as fully met.","Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.")</f>
+        <v>Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.</v>
       </c>
       <c r="H67" s="21" t="n"/>
       <c r="I67" s="67" t="str">
-        <f>IF('2. Assessment'!E29="","",'2. Assessment'!H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3")</f>
+        <f>IF('2. Assessment'!E29="","",'2. Assessment'!H29&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6")</f>
         <v/>
       </c>
       <c r="J67" s="21" t="n"/>
@@ -4544,9 +4544,9 @@
     <row r="68" ht="77.5" customHeight="1">
       <c r="B68" s="66" t="inlineStr">
         <is>
-          <t>Q20  Defending against AI-enabled threats
-AI Security &amp; Threat Risk
-AI Ready7: 7.1, 7.2, 7.3, 7.4, 7.5
+          <t>Q20  Model risk management &amp; validation
+Data &amp; Technology
+AI Ready7: 4.4, 6.3
 ☆ Recommended</t>
         </is>
       </c>
@@ -4558,12 +4558,12 @@
       <c r="E68" s="21" t="n"/>
       <c r="F68" s="21" t="n"/>
       <c r="G68" s="67" t="str">
-        <f>IF('2. Assessment'!F30=1,"N/A - reported as fully met.","Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.")</f>
-        <v>Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.</v>
+        <f>IF('2. Assessment'!F30=1,"N/A - reported as fully met.","Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.")</f>
+        <v>Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.</v>
       </c>
       <c r="H68" s="21" t="n"/>
       <c r="I68" s="67" t="str">
-        <f>IF('2. Assessment'!E30="","",'2. Assessment'!H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: AT-1, AT-2, AT-3, AT-4")</f>
+        <f>IF('2. Assessment'!E30="","",'2. Assessment'!H30&amp;CHAR(10)&amp;CHAR(10)&amp;"Controls: LC-9, RS-6, LC-13, OM-1")</f>
         <v/>
       </c>
       <c r="J68" s="21" t="n"/>
@@ -5463,7 +5463,7 @@
       </c>
       <c r="F112" s="62" t="inlineStr">
         <is>
-          <t>AI governance structure and policies, AI risk management framework and risk appetite, AI register, third-party AI risk, RCM-based compliance reviews, ISO/IEC 42001 readiness.</t>
+          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, RCM-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
         </is>
       </c>
       <c r="G112" s="21" t="n"/>
@@ -5475,7 +5475,7 @@
     <row r="113" ht="32" customHeight="1">
       <c r="B113" s="61" t="inlineStr">
         <is>
-          <t>AI Strategy &amp; Roadmap</t>
+          <t>AI Risk &amp; Cyber Resilience</t>
         </is>
       </c>
       <c r="C113" s="21" t="n"/>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="F113" s="62" t="inlineStr">
         <is>
-          <t>AI Opportunity Discovery (where AI and automation fit), AI strategy, use-case prioritisation, value-realisation KPIs and phased roadmap.</t>
+          <t>AI risk management framework and risk appetite, use-case risk &amp; impact assessments, third-party AI risk, AI security audits (GT AI Security &amp; Agent Audit Checklist), AI red teaming, deepfake-resilient processes.</t>
         </is>
       </c>
       <c r="G113" s="21" t="n"/>
@@ -5509,7 +5509,7 @@
       </c>
       <c r="F114" s="62" t="inlineStr">
         <is>
-          <t>AI literacy programmes, role-based pathways, immersive labs, deepfake &amp; AI-phishing simulations, board AI governance sessions.</t>
+          <t>AI literacy programmes (EU AI Act Art. 4-aligned), role-based pathways, immersive labs, deepfake &amp; AI-phishing simulations, board AI governance sessions.</t>
         </is>
       </c>
       <c r="G114" s="21" t="n"/>
@@ -5521,7 +5521,7 @@
     <row r="115" ht="32" customHeight="1">
       <c r="B115" s="61" t="inlineStr">
         <is>
-          <t>AI-Driven Automation &amp; Data</t>
+          <t>AI Strategy &amp; Roadmap</t>
         </is>
       </c>
       <c r="C115" s="21" t="n"/>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="F115" s="62" t="inlineStr">
         <is>
-          <t>Technology evaluation, data readiness, reference architecture, model validation and integration. GT AI apps in preparation: AI-powered BCP tool and AI-powered Financial Statements tool.</t>
+          <t>AI Opportunity Discovery (where AI and automation fit), AI strategy, use-case prioritisation, value-realisation KPIs and phased roadmap.</t>
         </is>
       </c>
       <c r="G115" s="21" t="n"/>
@@ -5544,7 +5544,7 @@
     <row r="116" ht="32" customHeight="1">
       <c r="B116" s="61" t="inlineStr">
         <is>
-          <t>AI Security &amp; Cyber Resilience</t>
+          <t>AI-Driven Automation &amp; Data</t>
         </is>
       </c>
       <c r="C116" s="21" t="n"/>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="F116" s="62" t="inlineStr">
         <is>
-          <t>AI security audits (GT AI Security &amp; Agent Audit Checklist), AI red teaming, secure AI agents, deepfake-resilient processes.</t>
+          <t>Technology evaluation, data readiness, reference architecture, model validation and integration. GT AI apps in preparation: AI-powered BCP tool and AI-powered Financial Statements tool.</t>
         </is>
       </c>
       <c r="G116" s="21" t="n"/>
@@ -6205,7 +6205,7 @@
   </conditionalFormatting>
   <printOptions horizontalCentered="0" gridLines="0"/>
   <pageMargins left="0.45" right="0.45" top="0.6" bottom="0.6" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1"/>
   <headerFooter>
     <oddHeader/>
     <oddFooter>&amp;L&amp;8 GT AI Readiness &amp;&amp; Risk Assessment - Confidential&amp;R&amp;8 Page &amp;P</oddFooter>
@@ -6214,12 +6214,13 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="5" manualBreakCount="5">
-    <brk id="29" min="0" max="16383" man="1"/>
-    <brk id="54" min="0" max="16383" man="1"/>
-    <brk id="64" min="0" max="16383" man="1"/>
-    <brk id="83" min="0" max="16383" man="1"/>
-    <brk id="104" min="0" max="16383" man="1"/>
+  <rowBreaks count="6" manualBreakCount="6">
+    <brk id="24" min="0" max="16383" man="1"/>
+    <brk id="50" min="0" max="16383" man="1"/>
+    <brk id="61" min="0" max="16383" man="1"/>
+    <brk id="75" min="0" max="16383" man="1"/>
+    <brk id="97" min="0" max="16383" man="1"/>
+    <brk id="117" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -6329,8 +6330,8 @@
       </c>
       <c r="C5" s="61" t="inlineStr">
         <is>
-          <t>AI strategy &amp; executive ownership
-(Strategy &amp; Value)</t>
+          <t>AI governance structure &amp; accountability
+(AI Governance)</t>
         </is>
       </c>
       <c r="D5" s="37" t="str">
@@ -6351,7 +6352,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>GL-1, GL-3</t>
+          <t>GL-1, GL-2, GL-7, AA-1</t>
         </is>
       </c>
       <c r="I5" s="6" t="n"/>
@@ -6367,8 +6368,8 @@
       </c>
       <c r="C6" s="61" t="inlineStr">
         <is>
-          <t>Use-case portfolio &amp; value realisation
-(Strategy &amp; Value)</t>
+          <t>AI policy, acceptable use &amp; regulatory compliance
+(AI Governance)</t>
         </is>
       </c>
       <c r="D6" s="37" t="str">
@@ -6389,7 +6390,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>GL-6, GL-5</t>
+          <t>GL-5, RO-1, RO-5</t>
         </is>
       </c>
       <c r="I6" s="6" t="n"/>
@@ -6405,8 +6406,8 @@
       </c>
       <c r="C7" s="61" t="inlineStr">
         <is>
-          <t>AI governance structure &amp; accountability
-(Governance, Risk &amp; Compliance)</t>
+          <t>Responsible-AI guardrails &amp; human oversight
+(AI Governance)</t>
         </is>
       </c>
       <c r="D7" s="37" t="str">
@@ -6427,7 +6428,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>GL-1, GL-2, GL-7, AA-1</t>
+          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -6443,8 +6444,8 @@
       </c>
       <c r="C8" s="61" t="inlineStr">
         <is>
-          <t>AI policy, acceptable use &amp; regulatory compliance
-(Governance, Risk &amp; Compliance)</t>
+          <t>AI incidents, monitoring &amp; assurance
+(AI Governance)</t>
         </is>
       </c>
       <c r="D8" s="37" t="str">
@@ -6465,7 +6466,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>GL-5, RO-1, RO-5</t>
+          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
         </is>
       </c>
       <c r="I8" s="6" t="n"/>
@@ -6482,7 +6483,7 @@
       <c r="C9" s="61" t="inlineStr">
         <is>
           <t>AI risk management framework
-(Governance, Risk &amp; Compliance)</t>
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D9" s="37" t="str">
@@ -6520,7 +6521,7 @@
       <c r="C10" s="61" t="inlineStr">
         <is>
           <t>AI risk appetite, KRIs &amp; reporting
-(Governance, Risk &amp; Compliance)</t>
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D10" s="37" t="str">
@@ -6558,7 +6559,7 @@
       <c r="C11" s="61" t="inlineStr">
         <is>
           <t>AI inventory &amp; risk / impact assessment
-(Governance, Risk &amp; Compliance)</t>
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D11" s="37" t="str">
@@ -6596,7 +6597,7 @@
       <c r="C12" s="61" t="inlineStr">
         <is>
           <t>Third-party &amp; AI supply-chain risk
-(Governance, Risk &amp; Compliance)</t>
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D12" s="37" t="str">
@@ -6633,8 +6634,8 @@
       </c>
       <c r="C13" s="61" t="inlineStr">
         <is>
-          <t>Responsible-AI guardrails &amp; human oversight
-(Governance, Risk &amp; Compliance)</t>
+          <t>Securing AI systems
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D13" s="37" t="str">
@@ -6655,7 +6656,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
+          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
@@ -6671,8 +6672,8 @@
       </c>
       <c r="C14" s="61" t="inlineStr">
         <is>
-          <t>AI incidents, monitoring &amp; assurance
-(Governance, Risk &amp; Compliance)</t>
+          <t>Defending against AI-enabled threats
+(AI Risk &amp; Security)</t>
         </is>
       </c>
       <c r="D14" s="37" t="str">
@@ -6693,7 +6694,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
+          <t>AT-1, AT-2, AT-3, AT-4</t>
         </is>
       </c>
       <c r="I14" s="6" t="n"/>
@@ -6709,8 +6710,8 @@
       </c>
       <c r="C15" s="61" t="inlineStr">
         <is>
-          <t>AI literacy &amp; capability
-(People &amp; Skills)</t>
+          <t>AI training, literacy &amp; awareness
+(Training &amp; Awareness)</t>
         </is>
       </c>
       <c r="D15" s="37" t="str">
@@ -6747,8 +6748,8 @@
       </c>
       <c r="C16" s="61" t="inlineStr">
         <is>
-          <t>Data governance, quality &amp; privacy for AI
-(Data &amp; Technology)</t>
+          <t>AI strategy &amp; executive ownership
+(Strategy &amp; Value)</t>
         </is>
       </c>
       <c r="D16" s="37" t="str">
@@ -6769,7 +6770,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
+          <t>GL-1, GL-3</t>
         </is>
       </c>
       <c r="I16" s="6" t="n"/>
@@ -6785,8 +6786,8 @@
       </c>
       <c r="C17" s="61" t="inlineStr">
         <is>
-          <t>AI architecture, integration &amp; monitoring
-(Data &amp; Technology)</t>
+          <t>Use-case portfolio &amp; value realisation
+(Strategy &amp; Value)</t>
         </is>
       </c>
       <c r="D17" s="37" t="str">
@@ -6807,7 +6808,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
+          <t>GL-6, GL-5</t>
         </is>
       </c>
       <c r="I17" s="6" t="n"/>
@@ -6823,7 +6824,7 @@
       </c>
       <c r="C18" s="61" t="inlineStr">
         <is>
-          <t>Model risk management &amp; validation
+          <t>Data governance, quality &amp; privacy for AI
 (Data &amp; Technology)</t>
         </is>
       </c>
@@ -6845,7 +6846,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>LC-9, RS-6, LC-13, OM-1</t>
+          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
         </is>
       </c>
       <c r="I18" s="6" t="n"/>
@@ -6861,8 +6862,8 @@
       </c>
       <c r="C19" s="61" t="inlineStr">
         <is>
-          <t>Securing AI systems
-(AI Security &amp; Threat Risk)</t>
+          <t>AI architecture, integration &amp; monitoring
+(Data &amp; Technology)</t>
         </is>
       </c>
       <c r="D19" s="37" t="str">
@@ -6883,7 +6884,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
+          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
         </is>
       </c>
       <c r="I19" s="6" t="n"/>
@@ -6899,8 +6900,8 @@
       </c>
       <c r="C20" s="61" t="inlineStr">
         <is>
-          <t>Defending against AI-enabled threats
-(AI Security &amp; Threat Risk)</t>
+          <t>Model risk management &amp; validation
+(Data &amp; Technology)</t>
         </is>
       </c>
       <c r="D20" s="37" t="str">
@@ -6921,7 +6922,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>AT-1, AT-2, AT-3, AT-4</t>
+          <t>LC-9, RS-6, LC-13, OM-1</t>
         </is>
       </c>
       <c r="I20" s="6" t="n"/>
@@ -6986,11 +6987,11 @@
       <c r="G3" s="21" t="n"/>
       <c r="H3" s="21" t="n"/>
     </row>
-    <row r="4" ht="71" customHeight="1">
+    <row r="4" ht="84" customHeight="1">
       <c r="B4" s="81" t="inlineStr">
         <is>
           <t>1) NSW AI Assessment Framework (AIAF, Digital NSW): lifecycle triggers, inherent-risk questions (AI use, decision impact, data, autonomy / reversibility), Low-Critical risk bands, pattern overrides, oversight pathways and the 8 ethics principles.
-2) GT AI Ready7: the 7 pillars (33 items) are consolidated into 5 domains - Strategy &amp; Value; Governance, Risk &amp; Compliance; People &amp; Skills; Data &amp; Technology; AI Security &amp; Threat Risk - using the AI Ready7 maturity scale Partial / Informed / Repeatable / Adaptive.
+2) GT AI Ready7: the 7 pillars (33 items) are consolidated into 5 domains - AI Governance; AI Risk &amp; Security (Protect AI Systems + Protection from AI Threats, plus AI risk management); Training &amp; Awareness; Strategy &amp; Value; Data &amp; Technology - using the AI Ready7 maturity scale Partial / Informed / Repeatable / Adaptive.
 3) GT AI RCM v2.1: every readiness question is mapped to the controls that evidence it, so results convert directly into a control-remediation plan.</t>
         </is>
       </c>
@@ -7460,17 +7461,17 @@
       </c>
       <c r="C31" s="62" t="inlineStr">
         <is>
-          <t>AI strategy &amp; executive ownership</t>
+          <t>AI governance structure &amp; accountability</t>
         </is>
       </c>
       <c r="D31" s="62" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value (1.1)</t>
+          <t>AI Governance (1.1, 2.3)</t>
         </is>
       </c>
       <c r="E31" s="62" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="F31" s="62" t="inlineStr">
@@ -7480,7 +7481,7 @@
       </c>
       <c r="G31" s="62" t="inlineStr">
         <is>
-          <t>GL-1, GL-3</t>
+          <t>GL-1, GL-2, GL-7, AA-1</t>
         </is>
       </c>
       <c r="H31" s="62" t="inlineStr">
@@ -7497,27 +7498,27 @@
       </c>
       <c r="C32" s="62" t="inlineStr">
         <is>
-          <t>Use-case portfolio &amp; value realisation</t>
+          <t>AI policy, acceptable use &amp; regulatory compliance</t>
         </is>
       </c>
       <c r="D32" s="62" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value (1.2, 1.3)</t>
+          <t>AI Governance (2.1, 2.2)</t>
         </is>
       </c>
       <c r="E32" s="62" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="F32" s="62" t="inlineStr">
         <is>
-          <t>Human, Social &amp; Environmental Wellbeing</t>
+          <t>Accountability, Privacy &amp; Security</t>
         </is>
       </c>
       <c r="G32" s="62" t="inlineStr">
         <is>
-          <t>GL-6, GL-5</t>
+          <t>GL-5, RO-1, RO-5</t>
         </is>
       </c>
       <c r="H32" s="62" t="inlineStr">
@@ -7534,27 +7535,27 @@
       </c>
       <c r="C33" s="62" t="inlineStr">
         <is>
-          <t>AI governance structure &amp; accountability</t>
+          <t>Responsible-AI guardrails &amp; human oversight</t>
         </is>
       </c>
       <c r="D33" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (1.1, 2.3)</t>
+          <t>AI Governance (2.3, 5.2)</t>
         </is>
       </c>
       <c r="E33" s="62" t="inlineStr">
         <is>
-          <t>⚠ Mandatory Requirement</t>
+          <t>⚖ Ethical Consideration</t>
         </is>
       </c>
       <c r="F33" s="62" t="inlineStr">
         <is>
-          <t>Accountability</t>
+          <t>Fairness, Transparency &amp; Explainability, Human-Centred Values, Contestability</t>
         </is>
       </c>
       <c r="G33" s="62" t="inlineStr">
         <is>
-          <t>GL-1, GL-2, GL-7, AA-1</t>
+          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
         </is>
       </c>
       <c r="H33" s="62" t="inlineStr">
@@ -7571,12 +7572,12 @@
       </c>
       <c r="C34" s="62" t="inlineStr">
         <is>
-          <t>AI policy, acceptable use &amp; regulatory compliance</t>
+          <t>AI incidents, monitoring &amp; assurance</t>
         </is>
       </c>
       <c r="D34" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.1, 2.2)</t>
+          <t>AI Governance (2.2, 7.4)</t>
         </is>
       </c>
       <c r="E34" s="62" t="inlineStr">
@@ -7586,12 +7587,12 @@
       </c>
       <c r="F34" s="62" t="inlineStr">
         <is>
-          <t>Accountability, Privacy &amp; Security</t>
+          <t>Accountability, Reliability &amp; Safety, Contestability, Transparency &amp; Explainability</t>
         </is>
       </c>
       <c r="G34" s="62" t="inlineStr">
         <is>
-          <t>GL-5, RO-1, RO-5</t>
+          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
         </is>
       </c>
       <c r="H34" s="62" t="inlineStr">
@@ -7613,7 +7614,7 @@
       </c>
       <c r="D35" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.4)</t>
+          <t>AI Risk &amp; Security (2.4)</t>
         </is>
       </c>
       <c r="E35" s="62" t="inlineStr">
@@ -7650,7 +7651,7 @@
       </c>
       <c r="D36" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (1.1, 4.4)</t>
+          <t>AI Risk &amp; Security (1.1, 4.4)</t>
         </is>
       </c>
       <c r="E36" s="62" t="inlineStr">
@@ -7687,7 +7688,7 @@
       </c>
       <c r="D37" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.4, 2.5)</t>
+          <t>AI Risk &amp; Security (2.4, 2.5)</t>
         </is>
       </c>
       <c r="E37" s="62" t="inlineStr">
@@ -7724,7 +7725,7 @@
       </c>
       <c r="D38" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.4, 6.2)</t>
+          <t>AI Risk &amp; Security (2.4, 6.2)</t>
         </is>
       </c>
       <c r="E38" s="62" t="inlineStr">
@@ -7756,27 +7757,27 @@
       </c>
       <c r="C39" s="62" t="inlineStr">
         <is>
-          <t>Responsible-AI guardrails &amp; human oversight</t>
+          <t>Securing AI systems</t>
         </is>
       </c>
       <c r="D39" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.3, 5.2)</t>
+          <t>AI Risk &amp; Security (6.1, 6.2, 6.3, 6.4, 6.5)</t>
         </is>
       </c>
       <c r="E39" s="62" t="inlineStr">
         <is>
-          <t>⚖ Ethical Consideration</t>
+          <t>⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="F39" s="62" t="inlineStr">
         <is>
-          <t>Fairness, Transparency &amp; Explainability, Human-Centred Values, Contestability</t>
+          <t>Privacy &amp; Security, Reliability &amp; Safety</t>
         </is>
       </c>
       <c r="G39" s="62" t="inlineStr">
         <is>
-          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
+          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
         </is>
       </c>
       <c r="H39" s="62" t="inlineStr">
@@ -7793,27 +7794,27 @@
       </c>
       <c r="C40" s="62" t="inlineStr">
         <is>
-          <t>AI incidents, monitoring &amp; assurance</t>
+          <t>Defending against AI-enabled threats</t>
         </is>
       </c>
       <c r="D40" s="62" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance (2.2, 7.4)</t>
+          <t>AI Risk &amp; Security (7.1, 7.2, 7.3, 7.4, 7.5)</t>
         </is>
       </c>
       <c r="E40" s="62" t="inlineStr">
         <is>
-          <t>⟳ Compliance Obligation</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="F40" s="62" t="inlineStr">
         <is>
-          <t>Accountability, Reliability &amp; Safety, Contestability, Transparency &amp; Explainability</t>
+          <t>Privacy &amp; Security</t>
         </is>
       </c>
       <c r="G40" s="62" t="inlineStr">
         <is>
-          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
+          <t>AT-1, AT-2, AT-3, AT-4</t>
         </is>
       </c>
       <c r="H40" s="62" t="inlineStr">
@@ -7830,12 +7831,12 @@
       </c>
       <c r="C41" s="62" t="inlineStr">
         <is>
-          <t>AI literacy &amp; capability</t>
+          <t>AI training, literacy &amp; awareness</t>
         </is>
       </c>
       <c r="D41" s="62" t="inlineStr">
         <is>
-          <t>People &amp; Skills (3.1, 3.2, 3.3, 3.4)</t>
+          <t>Training &amp; Awareness (3.1, 3.2, 3.3, 3.4)</t>
         </is>
       </c>
       <c r="E41" s="62" t="inlineStr">
@@ -7867,27 +7868,27 @@
       </c>
       <c r="C42" s="62" t="inlineStr">
         <is>
-          <t>Data governance, quality &amp; privacy for AI</t>
+          <t>AI strategy &amp; executive ownership</t>
         </is>
       </c>
       <c r="D42" s="62" t="inlineStr">
         <is>
-          <t>Data &amp; Technology (5.1, 5.3, 5.4, 5.5)</t>
+          <t>Strategy &amp; Value (1.1)</t>
         </is>
       </c>
       <c r="E42" s="62" t="inlineStr">
         <is>
-          <t>⟳ Compliance Obligation</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="F42" s="62" t="inlineStr">
         <is>
-          <t>Privacy &amp; Security, Fairness</t>
+          <t>Accountability</t>
         </is>
       </c>
       <c r="G42" s="62" t="inlineStr">
         <is>
-          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
+          <t>GL-1, GL-3</t>
         </is>
       </c>
       <c r="H42" s="62" t="inlineStr">
@@ -7904,12 +7905,12 @@
       </c>
       <c r="C43" s="62" t="inlineStr">
         <is>
-          <t>AI architecture, integration &amp; monitoring</t>
+          <t>Use-case portfolio &amp; value realisation</t>
         </is>
       </c>
       <c r="D43" s="62" t="inlineStr">
         <is>
-          <t>Data &amp; Technology (4.1, 4.2, 4.3, 4.4, 4.5)</t>
+          <t>Strategy &amp; Value (1.2, 1.3)</t>
         </is>
       </c>
       <c r="E43" s="62" t="inlineStr">
@@ -7919,12 +7920,12 @@
       </c>
       <c r="F43" s="62" t="inlineStr">
         <is>
-          <t>Reliability &amp; Safety</t>
+          <t>Human, Social &amp; Environmental Wellbeing</t>
         </is>
       </c>
       <c r="G43" s="62" t="inlineStr">
         <is>
-          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
+          <t>GL-6, GL-5</t>
         </is>
       </c>
       <c r="H43" s="62" t="inlineStr">
@@ -7941,27 +7942,27 @@
       </c>
       <c r="C44" s="62" t="inlineStr">
         <is>
-          <t>Model risk management &amp; validation</t>
+          <t>Data governance, quality &amp; privacy for AI</t>
         </is>
       </c>
       <c r="D44" s="62" t="inlineStr">
         <is>
-          <t>Data &amp; Technology (4.4, 6.3)</t>
+          <t>Data &amp; Technology (5.1, 5.3, 5.4, 5.5)</t>
         </is>
       </c>
       <c r="E44" s="62" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="F44" s="62" t="inlineStr">
         <is>
-          <t>Reliability &amp; Safety, Fairness</t>
+          <t>Privacy &amp; Security, Fairness</t>
         </is>
       </c>
       <c r="G44" s="62" t="inlineStr">
         <is>
-          <t>LC-9, RS-6, LC-13, OM-1</t>
+          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
         </is>
       </c>
       <c r="H44" s="62" t="inlineStr">
@@ -7978,27 +7979,27 @@
       </c>
       <c r="C45" s="62" t="inlineStr">
         <is>
-          <t>Securing AI systems</t>
+          <t>AI architecture, integration &amp; monitoring</t>
         </is>
       </c>
       <c r="D45" s="62" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk (6.1, 6.2, 6.3, 6.4, 6.5)</t>
+          <t>Data &amp; Technology (4.1, 4.2, 4.3, 4.4, 4.5)</t>
         </is>
       </c>
       <c r="E45" s="62" t="inlineStr">
         <is>
-          <t>⚠ Mandatory Requirement</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="F45" s="62" t="inlineStr">
         <is>
-          <t>Privacy &amp; Security, Reliability &amp; Safety</t>
+          <t>Reliability &amp; Safety</t>
         </is>
       </c>
       <c r="G45" s="62" t="inlineStr">
         <is>
-          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
+          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
         </is>
       </c>
       <c r="H45" s="62" t="inlineStr">
@@ -8015,12 +8016,12 @@
       </c>
       <c r="C46" s="62" t="inlineStr">
         <is>
-          <t>Defending against AI-enabled threats</t>
+          <t>Model risk management &amp; validation</t>
         </is>
       </c>
       <c r="D46" s="62" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk (7.1, 7.2, 7.3, 7.4, 7.5)</t>
+          <t>Data &amp; Technology (4.4, 6.3)</t>
         </is>
       </c>
       <c r="E46" s="62" t="inlineStr">
@@ -8030,12 +8031,12 @@
       </c>
       <c r="F46" s="62" t="inlineStr">
         <is>
-          <t>Privacy &amp; Security</t>
+          <t>Reliability &amp; Safety, Fairness</t>
         </is>
       </c>
       <c r="G46" s="62" t="inlineStr">
         <is>
-          <t>AT-1, AT-2, AT-3, AT-4</t>
+          <t>LC-9, RS-6, LC-13, OM-1</t>
         </is>
       </c>
       <c r="H46" s="62" t="inlineStr">
@@ -8715,7 +8716,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>No AI strategy or executive owner; AI adoption is unplanned</t>
+          <t>No defined AI governance; decisions are made ad hoc by individual teams</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -8728,7 +8729,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Appoint an executive AI sponsor and commission an AI strategy (situational / SWOT analysis, ambition, priority domains).</t>
+          <t>Appoint an executive AI owner and agree who decides on AI use cases; document interim responsibilities.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -8745,7 +8746,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Informal leadership interest; no documented strategy</t>
+          <t>Informal oversight by IT or a single function; roles not documented</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -8758,7 +8759,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Formalise leadership intent into a documented AI strategy approved by the executive committee.</t>
+          <t>Establish an AI committee / centre of excellence with a charter, decision rights and members from business, risk, legal, privacy and IT.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -8775,7 +8776,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Executive sponsor named and AI strategy drafted, but not linked to business objectives or budget</t>
+          <t>AI committee or sponsor defined on paper; roles and decision rights partly documented</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -8788,7 +8789,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Link the strategy to business objectives and budget; define experimentation ('sandbox') boundaries and communicate them.</t>
+          <t>Assign named business and technical owners to every AI system and publish a RACI across the three lines of defence.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -8805,7 +8806,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Approved AI strategy with executive ownership, priorities, budget and experimentation boundaries communicated to staff</t>
+          <t>Board / ExCo oversight, AI committee with charter and decision rights, named system owners and a documented RACI across the three lines</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -8818,7 +8819,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Track the strategy through KPIs and introduce an annual board-level review.</t>
+          <t>Introduce regular board / ExCo AI reporting and an annual governance-effectiveness review by internal audit.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -8835,7 +8836,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Strategy reviewed at least annually by the board, linked to business strategy and tracked through KPIs</t>
+          <t>Governance operates effectively: regular board reporting, periodic effectiveness review and independent assurance by internal audit</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -8848,7 +8849,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sustain: benchmark annually against peers and refresh the strategy as AI capabilities and regulation evolve.</t>
+          <t>Sustain: benchmark governance against ISO/IEC 42001 and refresh roles as AI use evolves.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -8865,7 +8866,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>No process - AI initiatives start ad hoc and value is not tracked</t>
+          <t>No AI policy; applicable AI regulations have not been identified</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -8878,7 +8879,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Create an AI use-case intake and approval process; build an initial prioritised backlog.</t>
+          <t>Issue an interim AI acceptable-use policy immediately (approved tools, prohibited data, output verification) and identify applicable regulations.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -8895,7 +8896,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Some use cases discussed informally; business cases are rare</t>
+          <t>Informal guidance only (e.g., emails); obligations understood by a few individuals</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -8908,7 +8909,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Introduce a standard business-case template with value, feasibility, data-readiness and risk scoring.</t>
+          <t>Approve a formal AI policy; build an AI obligations register covering Bahrain PDPL, sector rules (e.g., CBB) and extraterritorial regimes (EU AI Act).</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -8925,7 +8926,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Use-case intake exists and initiatives are prioritised, but benefits are not systematically tracked</t>
+          <t>AI acceptable-use policy approved; regulatory obligations identified but not mapped to controls</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -8938,7 +8939,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Define benefit KPIs (financial and non-financial) at approval and assign benefit owners.</t>
+          <t>Map each obligation to controls and owners using the GT AI RCM; require annual staff acknowledgement.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -8955,7 +8956,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Structured intake and prioritisation by value, feasibility, data readiness and risk; KPIs tracked for major initiatives</t>
+          <t>AI policy enforced with staff acknowledgement; obligations register maps regulations to controls and owners</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -8968,7 +8969,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Run quarterly portfolio reviews with continue / pivot / stop decisions; convert discovered shadow AI into governed use cases.</t>
+          <t>Establish monthly regulatory horizon scanning and periodic compliance testing with evidence retention.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -8985,7 +8986,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Portfolio managed as a whole with quarterly value / risk reviews, stop-or-scale decisions, and shadow-AI demand routed into the governed pipeline</t>
+          <t>Policy and obligations register reviewed regularly with horizon scanning; compliance tested and audit-ready evidence maintained</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -8998,7 +8999,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sustain: publish realised value to leadership and reinvest in proven use cases.</t>
+          <t>Sustain: keep audit-ready evidence packs and consider ISO/IEC 42001 certification.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -9015,7 +9016,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>No defined AI governance; decisions are made ad hoc by individual teams</t>
+          <t>No responsible-AI guardrails or oversight body</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -9028,7 +9029,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Appoint an executive AI owner and agree who decides on AI use cases; document interim responsibilities.</t>
+          <t>Establish an AI committee / centre of excellence with a charter and decision rights.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -9045,7 +9046,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Informal oversight by IT or a single function; roles not documented</t>
+          <t>High-level ethical principles published but not operationalised</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -9058,7 +9059,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Establish an AI committee / centre of excellence with a charter, decision rights and members from business, risk, legal, privacy and IT.</t>
+          <t>Translate ethical principles (GCC AI Ethics Manual, OECD) into practical guardrails: permitted uses, disclosure, human review, bias checks.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -9075,7 +9076,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AI committee or sponsor defined on paper; roles and decision rights partly documented</t>
+          <t>AI committee / CoE established; guardrails defined for some areas (e.g., human review of outputs)</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -9088,7 +9089,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assign named business and technical owners to every AI system and publish a RACI across the three lines of defence.</t>
+          <t>Apply mandatory human-in-charge controls and AI disclosure to all relevant AI; require committee approval for High / Critical uses.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -9105,7 +9106,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Board / ExCo oversight, AI committee with charter and decision rights, named system owners and a documented RACI across the three lines</t>
+          <t>Guardrails for fairness, transparency, disclosure and human-in-charge controls applied to all relevant AI; committee approves high-risk uses</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -9118,7 +9119,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Introduce regular board / ExCo AI reporting and an annual governance-effectiveness review by internal audit.</t>
+          <t>Test guardrail effectiveness (bias testing, oversight reviews) and provide contest / appeal routes for affected persons.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -9135,7 +9136,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Governance operates effectively: regular board reporting, periodic effectiveness review and independent assurance by internal audit</t>
+          <t>Guardrails tested (bias testing, oversight effectiveness); contestability routes for affected persons; lessons fed back into standards</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -9148,7 +9149,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sustain: benchmark governance against ISO/IEC 42001 and refresh roles as AI use evolves.</t>
+          <t>Sustain: publish a responsible-AI statement and report guardrail performance to the board.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -9165,7 +9166,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>No AI policy; applicable AI regulations have not been identified</t>
+          <t>No AI incident process or assurance</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -9178,7 +9179,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Issue an interim AI acceptable-use policy immediately (approved tools, prohibited data, output verification) and identify applicable regulations.</t>
+          <t>Define AI incident categories, severity and escalation within the existing incident process.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -9195,7 +9196,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Informal guidance only (e.g., emails); obligations understood by a few individuals</t>
+          <t>AI issues handled through general IT incident processes; no AI-specific assurance</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -9208,7 +9209,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Approve a formal AI policy; build an AI obligations register covering Bahrain PDPL, sector rules (e.g., CBB) and extraterritorial regimes (EU AI Act).</t>
+          <t>Add regulatory notification criteria (PDPL, CBB, EU AI Act Art. 73 where applicable) and AI incident logging.</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -9225,7 +9226,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>AI acceptable-use policy approved; regulatory obligations identified but not mapped to controls</t>
+          <t>AI incident categories and escalation defined; ad hoc reviews of AI controls</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -9238,7 +9239,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Map each obligation to controls and owners using the GT AI RCM; require annual staff acknowledgement.</t>
+          <t>Include AI governance in the internal-audit plan and obtain assurance evidence from AI vendors.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -9255,7 +9256,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>AI policy enforced with staff acknowledgement; obligations register maps regulations to controls and owners</t>
+          <t>AI incident management with regulatory notification criteria; periodic internal audit of AI governance; assurance obtained from AI vendors</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -9268,7 +9269,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Establish monthly regulatory horizon scanning and periodic compliance testing with evidence retention.</t>
+          <t>Implement post-incident learning and an ISO/IEC 42001 certification-readiness review.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -9285,7 +9286,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Policy and obligations register reviewed regularly with horizon scanning; compliance tested and audit-ready evidence maintained</t>
+          <t>Post-incident learning drives improvement; AI management system certified or certification-ready (ISO/IEC 42001); assurance reported to the board</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -9298,7 +9299,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sustain: keep audit-ready evidence packs and consider ISO/IEC 42001 certification.</t>
+          <t>Sustain: maintain certification and report AI assurance results to the board annually.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -9915,7 +9916,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>No responsible-AI guardrails or oversight body</t>
+          <t>AI systems are not specifically considered in security controls</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -9928,7 +9929,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Establish an AI committee / centre of excellence with a charter and decision rights.</t>
+          <t>Perform AI threat modelling (OWASP LLM Top 10) on existing AI systems and close critical exposures.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -9945,7 +9946,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>High-level ethical principles published but not operationalised</t>
+          <t>Standard IT security controls apply; no AI-specific threat assessment</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -9958,7 +9959,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Translate ethical principles (GCC AI Ethics Manual, OECD) into practical guardrails: permitted uses, disclosure, human review, bias checks.</t>
+          <t>Extend secure-development and access-management standards to AI, including non-human (agent) identities.</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -9975,7 +9976,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>AI committee / CoE established; guardrails defined for some areas (e.g., human review of outputs)</t>
+          <t>AI-specific threats (e.g., prompt injection, data leakage) assessed for some systems; access controls and logging in place</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -9988,7 +9989,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Apply mandatory human-in-charge controls and AI disclosure to all relevant AI; require committee approval for High / Critical uses.</t>
+          <t>Introduce AI red teaming before release, runtime guardrails (input / output filtering) and audit logging.</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -10005,7 +10006,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Guardrails for fairness, transparency, disclosure and human-in-charge controls applied to all relevant AI; committee approves high-risk uses</t>
+          <t>Secure AI development lifecycle; least privilege for users, systems and agents; sandboxed tool execution; AI red teaming before release; runtime guardrails and audit logging</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -10018,7 +10019,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Test guardrail effectiveness (bias testing, oversight reviews) and provide contest / appeal routes for affected persons.</t>
+          <t>Add AI supply-chain controls (model scanning, AI-BOM) and continuous adversarial testing integrated with the SOC.</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -10035,7 +10036,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Guardrails tested (bias testing, oversight effectiveness); contestability routes for affected persons; lessons fed back into standards</t>
+          <t>Continuous adversarial testing, AI supply-chain assurance (model scanning, AI-BOM) and forensic-ready logging integrated with the SOC</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -10048,7 +10049,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Sustain: publish a responsible-AI statement and report guardrail performance to the board.</t>
+          <t>Sustain: track AI security KRIs and re-test after every material model or provider change.</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -10065,7 +10066,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>No AI incident process or assurance</t>
+          <t>AI-enabled threats not considered</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -10078,7 +10079,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Define AI incident categories, severity and escalation within the existing incident process.</t>
+          <t>Introduce mandatory call-back / out-of-band verification for payments and sensitive requests.</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -10095,7 +10096,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>AI issues handled through general IT incident processes; no AI-specific assurance</t>
+          <t>General awareness only; no specific controls</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -10108,7 +10109,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Add regulatory notification criteria (PDPL, CBB, EU AI Act Art. 73 where applicable) and AI incident logging.</t>
+          <t>Add AI-enabled attack scenarios to threat intelligence, awareness and phishing simulations.</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -10125,7 +10126,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AI incident categories and escalation defined; ad hoc reviews of AI controls</t>
+          <t>Threat intelligence covers AI-enabled attacks; out-of-band verification for some high-risk requests</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -10138,7 +10139,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Include AI governance in the internal-audit plan and obtain assurance evidence from AI vendors.</t>
+          <t>Deploy behaviour-based detection and exercise AI incident playbooks (deepfake fraud, agent compromise).</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -10155,7 +10156,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AI incident management with regulatory notification criteria; periodic internal audit of AI governance; assurance obtained from AI vendors</t>
+          <t>Deepfake-resilient verification for payments and sensitive requests; behaviour-based detection; AI incident playbooks exercised</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -10168,7 +10169,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Implement post-incident learning and an ISO/IEC 42001 certification-readiness review.</t>
+          <t>Adopt continuous exposure management and AI-specific red teaming; reduce patch cycles to days.</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -10185,7 +10186,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Post-incident learning drives improvement; AI management system certified or certification-ready (ISO/IEC 42001); assurance reported to the board</t>
+          <t>Continuous exposure management and AI-specific red teaming; automated response at machine speed; critical vulnerabilities remediated in days</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -10198,7 +10199,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Sustain: maintain certification and report AI assurance results to the board annually.</t>
+          <t>Sustain: share AI threat intelligence with sector peers and national CERT.</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -10365,7 +10366,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Data used by AI is not classified or controlled; privacy requirements not considered</t>
+          <t>No AI strategy or executive owner; AI adoption is unplanned</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -10378,7 +10379,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Prohibit confidential / personal data in unapproved AI tools and apply data classification to AI use immediately.</t>
+          <t>Appoint an executive AI sponsor and commission an AI strategy (situational / SWOT analysis, ambition, priority domains).</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -10395,7 +10396,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Data classification policy exists but is not applied to AI; privacy reviewed case by case</t>
+          <t>Informal leadership interest; no documented strategy</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -10408,7 +10409,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Embed DPIAs for AI processing personal data and enforce classification-based handling rules (DLP).</t>
+          <t>Formalise leadership intent into a documented AI strategy approved by the executive committee.</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -10425,7 +10426,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Classification and handling rules apply to AI; DPIAs performed for some AI using personal data</t>
+          <t>Executive sponsor named and AI strategy drafted, but not linked to business objectives or budget</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -10438,7 +10439,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Require data-readiness assessments before approving use cases; implement minimisation, anonymisation and prompt redaction.</t>
+          <t>Link the strategy to business objectives and budget; define experimentation ('sandbox') boundaries and communicate them.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -10455,7 +10456,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Data readiness assessed before approval; lineage and quality monitored; minimisation, anonymisation and prompt redaction applied; DPIAs standard</t>
+          <t>Approved AI strategy with executive ownership, priorities, budget and experimentation boundaries communicated to staff</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -10468,7 +10469,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Automate data-quality and lineage monitoring; operationalise data-subject rights and transfer assessments for AI.</t>
+          <t>Track the strategy through KPIs and introduce an annual board-level review.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -10485,7 +10486,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Automated quality, lineage and privacy controls across AI pipelines; data-subject rights and cross-border transfers handled for AI systems</t>
+          <t>Strategy reviewed at least annually by the board, linked to business strategy and tracked through KPIs</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -10498,7 +10499,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Sustain: continuous data-quality KPIs and periodic privacy audits of AI systems.</t>
+          <t>Sustain: benchmark annually against peers and refresh the strategy as AI capabilities and regulation evolve.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -10515,7 +10516,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>No architectural standards; AI solutions built or bought in isolation</t>
+          <t>No process - AI initiatives start ad hoc and value is not tracked</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10528,7 +10529,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Define approved AI platforms and a minimum architecture standard (identity, data, logging) for all AI solutions.</t>
+          <t>Create an AI use-case intake and approval process; build an initial prioritised backlog.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -10545,7 +10546,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Some technical guidance exists; monitoring limited to availability</t>
+          <t>Some use cases discussed informally; business cases are rare</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10558,7 +10559,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Develop an enterprise AI reference architecture covering data, models, agents, integration and security.</t>
+          <t>Introduce a standard business-case template with value, feasibility, data-readiness and risk scoring.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -10575,7 +10576,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Reference architecture drafted; approved platforms and integration patterns for most AI; basic performance monitoring</t>
+          <t>Use-case intake exists and initiatives are prioritised, but benefits are not systematically tracked</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10588,7 +10589,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Centralise API / access control for AI, define agent execution authority and implement drift / performance monitoring with thresholds.</t>
+          <t>Define benefit KPIs (financial and non-financial) at approval and assign benefit owners.</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -10605,7 +10606,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Reference architecture adopted (data, models, agents, security); agent actions via a policy-enforcement gateway; performance, drift and bias monitored with thresholds; kill switches; cost governed</t>
+          <t>Structured intake and prioritisation by value, feasibility, data readiness and risk; KPIs tracked for major initiatives</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10618,7 +10619,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Implement KRI-based observability with automated responses and a governed pathway from citizen development to production.</t>
+          <t>Run quarterly portfolio reviews with continue / pivot / stop decisions; convert discovered shadow AI into governed use cases.</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -10635,7 +10636,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Full observability with KRIs and automated responses; governed path from citizen-developed AI to production; platform and vendor dependencies actively managed</t>
+          <t>Portfolio managed as a whole with quarterly value / risk reviews, stop-or-scale decisions, and shadow-AI demand routed into the governed pipeline</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10648,7 +10649,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Sustain: review architecture annually against emerging AI capabilities and vendor landscape.</t>
+          <t>Sustain: publish realised value to leadership and reinvest in proven use cases.</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -10665,7 +10666,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Models are not validated or inventoried</t>
+          <t>Data used by AI is not classified or controlled; privacy requirements not considered</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10678,7 +10679,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Create an inventory of AI / ML models and identify those that drive material decisions.</t>
+          <t>Prohibit confidential / personal data in unapproved AI tools and apply data classification to AI use immediately.</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -10695,7 +10696,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Developers test their own models; no independent review</t>
+          <t>Data classification policy exists but is not applied to AI; privacy reviewed case by case</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10708,7 +10709,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Introduce a model risk policy and require independent review (separate from developers) for material models.</t>
+          <t>Embed DPIAs for AI processing personal data and enforce classification-based handling rules (DLP).</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -10725,7 +10726,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Model inventory exists; validation performed for some material models</t>
+          <t>Classification and handling rules apply to AI; DPIAs performed for some AI using personal data</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10738,7 +10739,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Validate all material models before use and on a risk-based cycle; document thresholds, limitations and conditions of use.</t>
+          <t>Require data-readiness assessments before approving use cases; implement minimisation, anonymisation and prompt redaction.</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -10755,7 +10756,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Independent validation before use and on a risk-based cycle; performance thresholds and limitations documented</t>
+          <t>Data readiness assessed before approval; lineage and quality monitored; minimisation, anonymisation and prompt redaction applied; DPIAs standard</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10768,7 +10769,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Monitor model performance continuously and track validation findings to closure.</t>
+          <t>Automate data-quality and lineage monitoring; operationalise data-subject rights and transfer assessments for AI.</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -10785,7 +10786,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Model risk management aligned to SR 11-7 / PRA SS1/23 principles, with continuous monitoring and findings tracked to closure</t>
+          <t>Automated quality, lineage and privacy controls across AI pipelines; data-subject rights and cross-border transfers handled for AI systems</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10798,7 +10799,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Sustain: align with SR 11-7 / PRA SS1/23 principles and report model risk to the risk committee.</t>
+          <t>Sustain: continuous data-quality KPIs and periodic privacy audits of AI systems.</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -10815,7 +10816,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>AI systems are not specifically considered in security controls</t>
+          <t>No architectural standards; AI solutions built or bought in isolation</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -10828,7 +10829,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Perform AI threat modelling (OWASP LLM Top 10) on existing AI systems and close critical exposures.</t>
+          <t>Define approved AI platforms and a minimum architecture standard (identity, data, logging) for all AI solutions.</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -10845,7 +10846,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Standard IT security controls apply; no AI-specific threat assessment</t>
+          <t>Some technical guidance exists; monitoring limited to availability</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -10858,7 +10859,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Extend secure-development and access-management standards to AI, including non-human (agent) identities.</t>
+          <t>Develop an enterprise AI reference architecture covering data, models, agents, integration and security.</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -10875,7 +10876,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>AI-specific threats (e.g., prompt injection, data leakage) assessed for some systems; access controls and logging in place</t>
+          <t>Reference architecture drafted; approved platforms and integration patterns for most AI; basic performance monitoring</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -10888,7 +10889,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Introduce AI red teaming before release, runtime guardrails (input / output filtering) and audit logging.</t>
+          <t>Centralise API / access control for AI, define agent execution authority and implement drift / performance monitoring with thresholds.</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -10905,7 +10906,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Secure AI development lifecycle; least privilege for users, systems and agents; sandboxed tool execution; AI red teaming before release; runtime guardrails and audit logging</t>
+          <t>Reference architecture adopted (data, models, agents, security); agent actions via a policy-enforcement gateway; performance, drift and bias monitored with thresholds; kill switches; cost governed</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -10918,7 +10919,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Add AI supply-chain controls (model scanning, AI-BOM) and continuous adversarial testing integrated with the SOC.</t>
+          <t>Implement KRI-based observability with automated responses and a governed pathway from citizen development to production.</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -10935,7 +10936,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Continuous adversarial testing, AI supply-chain assurance (model scanning, AI-BOM) and forensic-ready logging integrated with the SOC</t>
+          <t>Full observability with KRIs and automated responses; governed path from citizen-developed AI to production; platform and vendor dependencies actively managed</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -10948,7 +10949,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Sustain: track AI security KRIs and re-test after every material model or provider change.</t>
+          <t>Sustain: review architecture annually against emerging AI capabilities and vendor landscape.</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -10965,7 +10966,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>AI-enabled threats not considered</t>
+          <t>Models are not validated or inventoried</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -10978,7 +10979,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Introduce mandatory call-back / out-of-band verification for payments and sensitive requests.</t>
+          <t>Create an inventory of AI / ML models and identify those that drive material decisions.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -10995,7 +10996,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>General awareness only; no specific controls</t>
+          <t>Developers test their own models; no independent review</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11008,7 +11009,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Add AI-enabled attack scenarios to threat intelligence, awareness and phishing simulations.</t>
+          <t>Introduce a model risk policy and require independent review (separate from developers) for material models.</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -11025,7 +11026,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Threat intelligence covers AI-enabled attacks; out-of-band verification for some high-risk requests</t>
+          <t>Model inventory exists; validation performed for some material models</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11038,7 +11039,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Deploy behaviour-based detection and exercise AI incident playbooks (deepfake fraud, agent compromise).</t>
+          <t>Validate all material models before use and on a risk-based cycle; document thresholds, limitations and conditions of use.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -11055,7 +11056,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Deepfake-resilient verification for payments and sensitive requests; behaviour-based detection; AI incident playbooks exercised</t>
+          <t>Independent validation before use and on a risk-based cycle; performance thresholds and limitations documented</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11068,7 +11069,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Adopt continuous exposure management and AI-specific red teaming; reduce patch cycles to days.</t>
+          <t>Monitor model performance continuously and track validation findings to closure.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -11085,7 +11086,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Continuous exposure management and AI-specific red teaming; automated response at machine speed; critical vulnerabilities remediated in days</t>
+          <t>Model risk management aligned to SR 11-7 / PRA SS1/23 principles, with continuous monitoring and findings tracked to closure</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -11098,7 +11099,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Sustain: share AI threat intelligence with sector peers and national CERT.</t>
+          <t>Sustain: align with SR 11-7 / PRA SS1/23 principles and report model risk to the risk committee.</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -11302,7 +11303,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="B37" t="str">
@@ -11318,12 +11319,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Without clear direction, ownership and value tracking, AI adoption is fragmented, duplicated and hard to justify, and risk-taking is unmanaged.</t>
+          <t>Without clear accountability, policy, oversight and assurance, AI is adopted inconsistently, misused and breaches regulation without anyone noticing or answering for it.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Governance</t>
         </is>
       </c>
       <c r="I37">
@@ -11337,7 +11338,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="B38" t="str">
@@ -11353,12 +11354,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Weak AI governance, risk management and compliance increase misuse, regulatory breaches, unmanaged third-party exposure and uncontrolled AI sprawl.</t>
+          <t>Without an AI risk framework, risk appetite, impact assessments, third-party controls and AI security, the organisation is exposed to unmanaged AI risk, prompt injection, data leakage, model compromise and deepfake-enabled fraud.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Governance &amp; Risk</t>
+          <t>Risk &amp; Security</t>
         </is>
       </c>
       <c r="I38">
@@ -11372,7 +11373,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>People &amp; Skills</t>
+          <t>Training &amp; Awareness</t>
         </is>
       </c>
       <c r="B39" t="str">
@@ -11388,12 +11389,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Low AI literacy and specialist capability increase unsafe use, susceptibility to AI-enabled threats and biased or unchecked outputs.</t>
+          <t>Low AI literacy and awareness increase unsafe use of AI tools, unchecked or biased outputs and susceptibility to AI-enabled phishing and deepfakes.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="I39">
@@ -11407,7 +11408,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="B40" t="str">
@@ -11423,12 +11424,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Weak data governance, architecture and model validation lead to inaccurate or biased outputs, privacy breaches, undetected drift and unsustainable costs.</t>
+          <t>Without clear direction, ownership and value tracking, AI adoption is fragmented, duplicated and hard to justify.</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Data &amp; Tech</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="I40">
@@ -11442,7 +11443,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="B41" t="str">
@@ -11458,12 +11459,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Weak AI security and threat defences expose the organisation to prompt injection, data leakage, model compromise and deepfake-enabled fraud.</t>
+          <t>Weak data governance, architecture and model validation lead to inaccurate or biased outputs, privacy breaches, undetected drift and unsustainable costs.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>AI Security</t>
+          <t>Data &amp; Tech</t>
         </is>
       </c>
       <c r="I41">
@@ -11839,12 +11840,12 @@
         </is>
       </c>
       <c r="B76" t="str">
-        <f>IFERROR(AVERAGE(E212,E215,E217),"")</f>
+        <f>IFERROR(AVERAGE(E206,E217,E219),"")</f>
         <v/>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Q13, Q16, Q18</t>
+          <t>Q7, Q18, Q20</t>
         </is>
       </c>
       <c r="D76" t="str">
@@ -11859,12 +11860,12 @@
         </is>
       </c>
       <c r="B77" t="str">
-        <f>IFERROR(AVERAGE(E207,E211,E215,E218,E219),"")</f>
+        <f>IFERROR(AVERAGE(E205,E211,E212,E213,E217),"")</f>
         <v/>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Q8, Q12, Q16, Q19, Q20</t>
+          <t>Q6, Q12, Q13, Q14, Q18</t>
         </is>
       </c>
       <c r="D77" t="str">
@@ -11879,12 +11880,12 @@
         </is>
       </c>
       <c r="B78" t="str">
-        <f>IFERROR(AVERAGE(E212,E213),"")</f>
+        <f>IFERROR(AVERAGE(E206,E207),"")</f>
         <v/>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Q13, Q14</t>
+          <t>Q7, Q8</t>
         </is>
       </c>
       <c r="D78" t="str">
@@ -11899,12 +11900,12 @@
         </is>
       </c>
       <c r="B79" t="str">
-        <f>IFERROR(AVERAGE(E204,E206,E207,E208,E209,E210,E211,E213),"")</f>
+        <f>IFERROR(AVERAGE(E204,E205,E207,E208,E209,E210,E211,E215),"")</f>
         <v/>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Q5, Q7, Q8, Q9, Q10, Q11, Q12, Q14</t>
+          <t>Q5, Q6, Q8, Q9, Q10, Q11, Q12, Q16</t>
         </is>
       </c>
       <c r="D79" t="str">
@@ -11919,12 +11920,12 @@
         </is>
       </c>
       <c r="B80" t="str">
-        <f>IFERROR(AVERAGE(E205,E210),"")</f>
+        <f>IFERROR(AVERAGE(E210,E216),"")</f>
         <v/>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Q6, Q11</t>
+          <t>Q11, Q17</t>
         </is>
       </c>
       <c r="D80" t="str">
@@ -11939,12 +11940,12 @@
         </is>
       </c>
       <c r="B81" t="str">
-        <f>IFERROR(AVERAGE(E212,E214),"")</f>
+        <f>IFERROR(AVERAGE(E206,E214),"")</f>
         <v/>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Q13, Q15</t>
+          <t>Q7, Q15</t>
         </is>
       </c>
       <c r="D81" t="str">
@@ -11959,12 +11960,12 @@
         </is>
       </c>
       <c r="B82" t="str">
-        <f>IFERROR(AVERAGE(E208,E213,E216,E217,E218),"")</f>
+        <f>IFERROR(AVERAGE(E207,E208,E212,E218,E219),"")</f>
         <v/>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Q9, Q14, Q17, Q18, Q19</t>
+          <t>Q8, Q9, Q13, Q19, Q20</t>
         </is>
       </c>
       <c r="D82" t="str">
@@ -11979,12 +11980,12 @@
         </is>
       </c>
       <c r="B83" t="str">
-        <f>IFERROR(AVERAGE(E212,E213),"")</f>
+        <f>IFERROR(AVERAGE(E206,E207),"")</f>
         <v/>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Q13, Q14</t>
+          <t>Q7, Q8</t>
         </is>
       </c>
       <c r="D83" t="str">
@@ -12225,16 +12226,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>AI governance structure and policies, AI risk management framework and risk appetite, AI register, third-party AI risk, RCM-based compliance reviews, ISO/IEC 42001 readiness.</t>
+          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, RCM-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
         </is>
       </c>
       <c r="D120" t="str">
-        <f>IFERROR(B38,"")</f>
+        <f>IFERROR(B37,"")</f>
         <v/>
       </c>
       <c r="E120" t="str">
@@ -12245,21 +12246,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>AI Strategy &amp; Roadmap</t>
+          <t>AI Risk &amp; Cyber Resilience</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>AI Opportunity Discovery (where AI and automation fit), AI strategy, use-case prioritisation, value-realisation KPIs and phased roadmap.</t>
+          <t>AI risk management framework and risk appetite, use-case risk &amp; impact assessments, third-party AI risk, AI security audits (GT AI Security &amp; Agent Audit Checklist), AI red teaming, deepfake-resilient processes.</t>
         </is>
       </c>
       <c r="D121" t="str">
-        <f>IFERROR(B37,"")</f>
+        <f>IFERROR(B38,"")</f>
         <v/>
       </c>
       <c r="E121" t="str">
@@ -12275,12 +12276,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>People &amp; Skills</t>
+          <t>Training &amp; Awareness</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>AI literacy programmes, role-based pathways, immersive labs, deepfake &amp; AI-phishing simulations, board AI governance sessions.</t>
+          <t>AI literacy programmes (EU AI Act Art. 4-aligned), role-based pathways, immersive labs, deepfake &amp; AI-phishing simulations, board AI governance sessions.</t>
         </is>
       </c>
       <c r="D122" t="str">
@@ -12295,17 +12296,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>AI-Driven Automation &amp; Data</t>
+          <t>AI Strategy &amp; Roadmap</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Technology evaluation, data readiness, reference architecture, model validation and integration. GT AI apps in preparation: AI-powered BCP tool and AI-powered Financial Statements tool.</t>
+          <t>AI Opportunity Discovery (where AI and automation fit), AI strategy, use-case prioritisation, value-realisation KPIs and phased roadmap.</t>
         </is>
       </c>
       <c r="D123" t="str">
@@ -12320,17 +12321,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>AI Security &amp; Cyber Resilience</t>
+          <t>AI-Driven Automation &amp; Data</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>AI security audits (GT AI Security &amp; Agent Audit Checklist), AI red teaming, secure AI agents, deepfake-resilient processes.</t>
+          <t>Technology evaluation, data readiness, reference architecture, model validation and integration. GT AI apps in preparation: AI-powered BCP tool and AI-powered Financial Statements tool.</t>
         </is>
       </c>
       <c r="D124" t="str">
@@ -12569,12 +12570,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>AI strategy &amp; executive ownership</t>
+          <t>AI governance structure &amp; accountability</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="D204">
@@ -12586,8 +12587,8 @@
         <v/>
       </c>
       <c r="F204">
-        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A204="Q7",A204="Q9",A204="Q11",A204="Q19")),0.5,0)</f>
-        <v>1</v>
+        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A204="Q7",A204="Q9",A204="Q11",A204="Q19")),0.5,0)</f>
+        <v>1.5</v>
       </c>
       <c r="G204" t="str">
         <f>IF(E204="","",1-E204)</f>
@@ -12615,12 +12616,12 @@
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>GL-1, GL-3</t>
+          <t>GL-1, GL-2, GL-7, AA-1</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="O204">
@@ -12633,7 +12634,7 @@
       </c>
       <c r="Q204" t="inlineStr">
         <is>
-          <t>Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.</t>
+          <t>Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.</t>
         </is>
       </c>
     </row>
@@ -12645,12 +12646,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Use-case portfolio &amp; value realisation</t>
+          <t>AI policy, acceptable use &amp; regulatory compliance</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Strategy &amp; Value</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="D205">
@@ -12662,8 +12663,8 @@
         <v/>
       </c>
       <c r="F205">
-        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A205="Q7",A205="Q9",A205="Q11",A205="Q19")),0.5,0)</f>
-        <v>1</v>
+        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A205="Q7",A205="Q9",A205="Q11",A205="Q19")),0.5,0)</f>
+        <v>1.5</v>
       </c>
       <c r="G205" t="str">
         <f>IF(E205="","",1-E205)</f>
@@ -12691,12 +12692,12 @@
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>GL-6, GL-5</t>
+          <t>GL-5, RO-1, RO-5</t>
         </is>
       </c>
       <c r="N205" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="O205">
@@ -12709,7 +12710,7 @@
       </c>
       <c r="Q205" t="inlineStr">
         <is>
-          <t>Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.</t>
+          <t>Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.</t>
         </is>
       </c>
     </row>
@@ -12721,12 +12722,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>AI governance structure &amp; accountability</t>
+          <t>Responsible-AI guardrails &amp; human oversight</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="D206">
@@ -12738,8 +12739,8 @@
         <v/>
       </c>
       <c r="F206">
-        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A206="Q7",A206="Q9",A206="Q11",A206="Q19")),0.5,0)</f>
-        <v>1.5</v>
+        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A206="Q7",A206="Q9",A206="Q11",A206="Q19")),0.5,0)</f>
+        <v>1</v>
       </c>
       <c r="G206" t="str">
         <f>IF(E206="","",1-E206)</f>
@@ -12767,12 +12768,12 @@
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>GL-1, GL-2, GL-7, AA-1</t>
+          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>⚠ Mandatory Requirement</t>
+          <t>⚖ Ethical Consideration</t>
         </is>
       </c>
       <c r="O206">
@@ -12785,7 +12786,7 @@
       </c>
       <c r="Q206" t="inlineStr">
         <is>
-          <t>Unclear accountability for AI decisions and outcomes, inconsistent approvals and no escalation route when AI fails.</t>
+          <t>Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.</t>
         </is>
       </c>
     </row>
@@ -12797,12 +12798,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>AI policy, acceptable use &amp; regulatory compliance</t>
+          <t>AI incidents, monitoring &amp; assurance</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Governance</t>
         </is>
       </c>
       <c r="D207">
@@ -12843,7 +12844,7 @@
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>GL-5, RO-1, RO-5</t>
+          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
         </is>
       </c>
       <c r="N207" t="inlineStr">
@@ -12861,7 +12862,7 @@
       </c>
       <c r="Q207" t="inlineStr">
         <is>
-          <t>Misuse of AI, data leakage and breach of legal or regulatory requirements, with exposure to penalties, licence conditions and reputational harm.</t>
+          <t>Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.</t>
         </is>
       </c>
     </row>
@@ -12878,7 +12879,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D208">
@@ -12954,7 +12955,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D209">
@@ -13030,7 +13031,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D210">
@@ -13106,7 +13107,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D211">
@@ -13177,12 +13178,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Responsible-AI guardrails &amp; human oversight</t>
+          <t>Securing AI systems</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D212">
@@ -13194,8 +13195,8 @@
         <v/>
       </c>
       <c r="F212">
-        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A212="Q7",A212="Q9",A212="Q11",A212="Q19")),0.5,0)</f>
-        <v>1</v>
+        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A212="Q7",A212="Q9",A212="Q11",A212="Q19")),0.5,0)</f>
+        <v>1.5</v>
       </c>
       <c r="G212" t="str">
         <f>IF(E212="","",1-E212)</f>
@@ -13223,12 +13224,12 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>GL-7, RS-1, RS-4, RS-5, CO-1, CO-3</t>
+          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>⚖ Ethical Consideration</t>
+          <t>⚠ Mandatory Requirement</t>
         </is>
       </c>
       <c r="O212">
@@ -13241,7 +13242,7 @@
       </c>
       <c r="Q212" t="inlineStr">
         <is>
-          <t>Biased or harmful outcomes, undisclosed AI use and lack of accountability for AI-supported decisions.</t>
+          <t>Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.</t>
         </is>
       </c>
     </row>
@@ -13253,12 +13254,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>AI incidents, monitoring &amp; assurance</t>
+          <t>Defending against AI-enabled threats</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Governance, Risk &amp; Compliance</t>
+          <t>AI Risk &amp; Security</t>
         </is>
       </c>
       <c r="D213">
@@ -13270,8 +13271,8 @@
         <v/>
       </c>
       <c r="F213">
-        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A213="Q7",A213="Q9",A213="Q11",A213="Q19")),0.5,0)</f>
-        <v>1.5</v>
+        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A213="Q7",A213="Q9",A213="Q11",A213="Q19")),0.5,0)</f>
+        <v>1</v>
       </c>
       <c r="G213" t="str">
         <f>IF(E213="","",1-E213)</f>
@@ -13299,12 +13300,12 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>IM-1, IM-2, IM-3, AA-1, AA-2, RO-4</t>
+          <t>AT-1, AT-2, AT-3, AT-4</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
         <is>
-          <t>⟳ Compliance Obligation</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="O213">
@@ -13317,7 +13318,7 @@
       </c>
       <c r="Q213" t="inlineStr">
         <is>
-          <t>Delayed response to AI failures, missed regulatory notifications and lack of defensible evidence for regulators, auditors and clients.</t>
+          <t>Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.</t>
         </is>
       </c>
     </row>
@@ -13329,12 +13330,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>AI literacy &amp; capability</t>
+          <t>AI training, literacy &amp; awareness</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>People &amp; Skills</t>
+          <t>Training &amp; Awareness</t>
         </is>
       </c>
       <c r="D214">
@@ -13405,12 +13406,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Data governance, quality &amp; privacy for AI</t>
+          <t>AI strategy &amp; executive ownership</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="D215">
@@ -13422,8 +13423,8 @@
         <v/>
       </c>
       <c r="F215">
-        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A215="Q7",A215="Q9",A215="Q11",A215="Q19")),0.5,0)</f>
-        <v>1.5</v>
+        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A215="Q7",A215="Q9",A215="Q11",A215="Q19")),0.5,0)</f>
+        <v>1</v>
       </c>
       <c r="G215" t="str">
         <f>IF(E215="","",1-E215)</f>
@@ -13451,12 +13452,12 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
+          <t>GL-1, GL-3</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>⟳ Compliance Obligation</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="O215">
@@ -13469,7 +13470,7 @@
       </c>
       <c r="Q215" t="inlineStr">
         <is>
-          <t>Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.</t>
+          <t>Lack of executive direction leads to inconsistent AI use, unmanaged risk-taking, poor-quality outputs and fragmented adoption.</t>
         </is>
       </c>
     </row>
@@ -13481,12 +13482,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>AI architecture, integration &amp; monitoring</t>
+          <t>Use-case portfolio &amp; value realisation</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Data &amp; Technology</t>
+          <t>Strategy &amp; Value</t>
         </is>
       </c>
       <c r="D216">
@@ -13527,7 +13528,7 @@
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
+          <t>GL-6, GL-5</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
@@ -13545,7 +13546,7 @@
       </c>
       <c r="Q216" t="inlineStr">
         <is>
-          <t>Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.</t>
+          <t>Duplicated or low-value AI investment, shadow AI and inability to demonstrate return on investment.</t>
         </is>
       </c>
     </row>
@@ -13557,7 +13558,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Model risk management &amp; validation</t>
+          <t>Data governance, quality &amp; privacy for AI</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -13574,8 +13575,8 @@
         <v/>
       </c>
       <c r="F217">
-        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A217="Q7",A217="Q9",A217="Q11",A217="Q19")),0.5,0)</f>
-        <v>1</v>
+        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A217="Q7",A217="Q9",A217="Q11",A217="Q19")),0.5,0)</f>
+        <v>1.5</v>
       </c>
       <c r="G217" t="str">
         <f>IF(E217="","",1-E217)</f>
@@ -13603,12 +13604,12 @@
       </c>
       <c r="M217" t="inlineStr">
         <is>
-          <t>LC-9, RS-6, LC-13, OM-1</t>
+          <t>LC-1, SE-4, PR-1, PR-4, PR-5, PR-6</t>
         </is>
       </c>
       <c r="N217" t="inlineStr">
         <is>
-          <t>☆ Recommended</t>
+          <t>⟳ Compliance Obligation</t>
         </is>
       </c>
       <c r="O217">
@@ -13621,7 +13622,7 @@
       </c>
       <c r="Q217" t="inlineStr">
         <is>
-          <t>Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.</t>
+          <t>Data breaches, PDPL non-compliance, and biased or inaccurate outputs from poor-quality or unsuitable data.</t>
         </is>
       </c>
     </row>
@@ -13633,12 +13634,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Securing AI systems</t>
+          <t>AI architecture, integration &amp; monitoring</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="D218">
@@ -13650,8 +13651,8 @@
         <v/>
       </c>
       <c r="F218">
-        <f>1.5+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A218="Q7",A218="Q9",A218="Q11",A218="Q19")),0.5,0)</f>
-        <v>1.5</v>
+        <f>1.0+IF(AND(OR(Calc!$C$32="High",Calc!$C$32="Critical"),OR(A218="Q7",A218="Q9",A218="Q11",A218="Q19")),0.5,0)</f>
+        <v>1</v>
       </c>
       <c r="G218" t="str">
         <f>IF(E218="","",1-E218)</f>
@@ -13679,12 +13680,12 @@
       </c>
       <c r="M218" t="inlineStr">
         <is>
-          <t>SE-2, SE-3, SE-6 to SE-10, OM-2, AA-3</t>
+          <t>LC-2, LC-3, LC-8, LC-12, OM-1, OM-4, RM-6</t>
         </is>
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t>⚠ Mandatory Requirement</t>
+          <t>☆ Recommended</t>
         </is>
       </c>
       <c r="O218">
@@ -13697,7 +13698,7 @@
       </c>
       <c r="Q218" t="inlineStr">
         <is>
-          <t>Unauthorised access, model compromise, data exfiltration through AI and undetected misuse.</t>
+          <t>Inconsistent and insecure implementations, undetected model drift or failure, excessive agent privileges and unsustainable AI costs.</t>
         </is>
       </c>
     </row>
@@ -13709,12 +13710,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Defending against AI-enabled threats</t>
+          <t>Model risk management &amp; validation</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>AI Security &amp; Threat Risk</t>
+          <t>Data &amp; Technology</t>
         </is>
       </c>
       <c r="D219">
@@ -13755,7 +13756,7 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>AT-1, AT-2, AT-3, AT-4</t>
+          <t>LC-9, RS-6, LC-13, OM-1</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
@@ -13773,7 +13774,7 @@
       </c>
       <c r="Q219" t="inlineStr">
         <is>
-          <t>Deepfake-enabled fraud, account compromise and faster, more scalable attacks that outpace defences.</t>
+          <t>Inaccurate, biased or unstable models drive decisions unnoticed, with regulatory exposure for financial-services clients.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Readiness proposal redesign; no Ready7 basis references; sector lens filled
- Readiness proposal: GT template icons, case-study visuals, staircase maturity curve with
  governance focus per stage, risks of lagging governance, client effort/output per day,
  domain 'if weak' panels, report previews, option 'best for' and report contents
- Removed references presenting GT AI Ready7 as the basis of the tool (report, proposal);
  Ready7 kept only as GT Bahrain's own results for comparison
- Sector lens / profiles: qualitative value statement for sectors not sized in the 2030 analysis

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
-          <t>MATURITY LEVEL (AI Ready7 scale)</t>
+          <t>MATURITY LEVEL</t>
         </is>
       </c>
       <c r="F4" s="23" t="inlineStr">
@@ -3283,7 +3283,7 @@
     </row>
     <row r="4">
       <c r="B4" s="44" t="str">
-        <f>IF(Calc!B21=1,"Framework basis: NSW AI Assessment Framework (inherent risk)  |  GT AI Ready7 (5 readiness domains)  |  GT AI RCM v2.1 (controls)  |  ISO/IEC 42001, NIST AI RMF, EU AI Act, Bahrain PDPL","ASSESSMENT INCOMPLETE - "&amp;Calc!B20&amp;" of 20 questions answered. Results below are provisional.")</f>
+        <f>IF(Calc!B21=1,"Framework basis: NSW AI Assessment Framework (inherent risk)  |  ISO/IEC 42001, ISO/IEC 23894, NIST AI RMF  |  EU AI Act, Bahrain PDPL  |  GT AI RCM v2.1 (controls)","ASSESSMENT INCOMPLETE - "&amp;Calc!B20&amp;" of 20 questions answered. Results below are provisional.")</f>
         <v>ASSESSMENT INCOMPLETE - 0 of 20 questions answered. Results below are provisional.</v>
       </c>
       <c r="M4" s="45" t="n"/>
@@ -3355,8 +3355,8 @@
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="B9" s="51" t="str">
-        <f>"AI Ready7 scale: &lt;50% Partial | 50-70% Informed | 70-90% Repeatable | 90%+ Adaptive"</f>
-        <v>AI Ready7 scale: &lt;50% Partial | 50-70% Informed | 70-90% Repeatable | 90%+ Adaptive</v>
+        <f>"Maturity scale: &lt;50% Partial | 50-70% Informed | 70-90% Repeatable | 90%+ Adaptive"</f>
+        <v>Maturity scale: &lt;50% Partial | 50-70% Informed | 70-90% Repeatable | 90%+ Adaptive</v>
       </c>
       <c r="C9" s="21" t="n"/>
       <c r="D9" s="21" t="n"/>
@@ -4126,7 +4126,6 @@
         <is>
           <t>Q5  AI governance structure &amp; accountability
 AI Governance
-AI Ready7: 1.1, 2.3
 ⚠ Mandatory Requirement</t>
         </is>
       </c>
@@ -4154,7 +4153,6 @@
         <is>
           <t>Q6  AI policy, acceptable use &amp; regulatory compliance
 AI Governance
-AI Ready7: 2.1, 2.2
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4182,7 +4180,6 @@
         <is>
           <t>Q7  Responsible-AI guardrails &amp; human oversight
 AI Governance
-AI Ready7: 2.3, 5.2
 ⚖ Ethical Consideration</t>
         </is>
       </c>
@@ -4210,7 +4207,6 @@
         <is>
           <t>Q8  AI incidents, monitoring &amp; assurance
 AI Governance
-AI Ready7: 2.2, 7.4
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4238,7 +4234,6 @@
         <is>
           <t>Q9  AI risk management framework
 AI Risk &amp; Security
-AI Ready7: 2.4
 ⚠ Mandatory Requirement</t>
         </is>
       </c>
@@ -4266,7 +4261,6 @@
         <is>
           <t>Q10  AI risk appetite, KRIs &amp; reporting
 AI Risk &amp; Security
-AI Ready7: 1.1, 4.4
 ⚠ Mandatory Requirement</t>
         </is>
       </c>
@@ -4294,7 +4288,6 @@
         <is>
           <t>Q11  AI inventory &amp; risk / impact assessment
 AI Risk &amp; Security
-AI Ready7: 2.4, 2.5
 ⚠ Mandatory Requirement</t>
         </is>
       </c>
@@ -4322,7 +4315,6 @@
         <is>
           <t>Q12  Third-party &amp; AI supply-chain risk
 AI Risk &amp; Security
-AI Ready7: 2.4, 6.2
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4350,7 +4342,6 @@
         <is>
           <t>Q13  Securing AI systems
 AI Risk &amp; Security
-AI Ready7: 6.1, 6.2, 6.3, 6.4, 6.5
 ⚠ Mandatory Requirement</t>
         </is>
       </c>
@@ -4378,7 +4369,6 @@
         <is>
           <t>Q14  Defending against AI-enabled threats
 AI Risk &amp; Security
-AI Ready7: 7.1, 7.2, 7.3, 7.4, 7.5
 ☆ Recommended</t>
         </is>
       </c>
@@ -4406,7 +4396,6 @@
         <is>
           <t>Q15  AI training, literacy &amp; awareness
 Training &amp; Awareness
-AI Ready7: 3.1, 3.2, 3.3, 3.4
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4434,7 +4423,6 @@
         <is>
           <t>Q16  AI strategy &amp; executive ownership
 Strategy &amp; Value
-AI Ready7: 1.1
 ☆ Recommended</t>
         </is>
       </c>
@@ -4462,7 +4450,6 @@
         <is>
           <t>Q17  Use-case portfolio &amp; value realisation
 Strategy &amp; Value
-AI Ready7: 1.2, 1.3
 ☆ Recommended</t>
         </is>
       </c>
@@ -4490,7 +4477,6 @@
         <is>
           <t>Q18  Data governance, quality &amp; privacy for AI
 Data &amp; Technology
-AI Ready7: 5.1, 5.3, 5.4, 5.5
 ⟳ Compliance Obligation</t>
         </is>
       </c>
@@ -4518,7 +4504,6 @@
         <is>
           <t>Q19  AI architecture, integration &amp; monitoring
 Data &amp; Technology
-AI Ready7: 4.1, 4.2, 4.3, 4.4, 4.5
 ☆ Recommended</t>
         </is>
       </c>
@@ -4546,7 +4531,6 @@
         <is>
           <t>Q20  Model risk management &amp; validation
 Data &amp; Technology
-AI Ready7: 4.4, 6.3
 ☆ Recommended</t>
         </is>
       </c>
@@ -5676,7 +5660,7 @@
     <row r="126" ht="58" customHeight="1">
       <c r="B126" s="78" t="inlineStr">
         <is>
-          <t>Methodology: Part A (4 questions) derives an inherent-risk tier from the NSW AI Assessment Framework risk factors (AI use, decision impact, data sensitivity, oversight &amp; reversibility). Part B (16 questions) scores readiness 0-100% across 5 domains derived from the GT AI Ready7 pillars; domain scores are averaged equally into the overall score and mapped to the AI Ready7 maturity scale. Exposure combines tier and maturity. Recommendations reference the GT AI RCM v2.1 controls.  Disclaimer: this is a self-assessment based on the responses provided and has not been independently verified by Grant Thornton. It is not an audit, certification or legal opinion.  (c) 2026 Grant Thornton Bahrain. All rights reserved.</t>
+          <t>Methodology: Part A (4 questions) derives an inherent-risk tier from the NSW AI Assessment Framework risk factors (AI use, decision impact, data sensitivity, oversight &amp; reversibility). Part B (16 questions) scores readiness 0-100% across 5 domains (AI Governance; AI Risk &amp; Security; Training &amp; Awareness; Strategy &amp; Value; Data &amp; Technology); domain scores are averaged equally into the overall score and mapped to a four-band maturity scale. Exposure combines tier and maturity. Recommendations reference the GT AI RCM v2.1 controls.  Disclaimer: this is a self-assessment based on the responses provided and has not been independently verified by Grant Thornton. It is not an audit, certification or legal opinion.  (c) 2026 Grant Thornton Bahrain. All rights reserved.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove RCM and version references from proposals and client report; unversioned file names
- Proposals (user's versions edited in place): controls referred to as the GT AI Risk Assessment
  Framework; no version numbers on GT tools or documents
- Client report and engine wording: controls of the GT AI Risk Assessment Framework (no RCM / v2.1)
- Toolkits, deck builders and app list updated to the same wording; report screenshots refreshed
- Files renamed: GT_AI_RCM.xlsx, GT_AI_Security_and_Agent_Audit_Checklist.xlsx,
  GT_AI_Risk_Assessment_Framework.docx

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8ossW6xvKTGEs2GV44CxS
</commit_message>
<xml_diff>
--- a/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
+++ b/01_AI_Governance_Risk_Compliance/1.3_AI_Readiness_Assessment_Tool/GT_AI_Readiness_Assessment_Tool.xlsx
@@ -1726,7 +1726,7 @@
     <row r="2" ht="44" customHeight="1">
       <c r="B2" s="22" t="inlineStr">
         <is>
-          <t>Select the statement in column E that best describes your current state (choose the lower level if unsure - evidence should exist for the level selected). Part A profiles your AI use and inherent risk (based on the NSW AI Assessment Framework). Part B measures readiness across 5 domains (derived from the 7 GT AI Ready7 pillars), mapped to the GT AI RCM v2.1 controls. Results update live below and in the '3. Report' sheet.</t>
+          <t>Select the statement in column E that best describes your current state (choose the lower level if unsure - evidence should exist for the level selected). Part A profiles your AI use and inherent risk (based on the NSW AI Assessment Framework). Part B measures readiness across 5 domains (derived from the 7 GT AI Ready7 pillars), mapped to the GT AI Risk Assessment Framework controls. Results update live below and in the '3. Report' sheet.</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="I8" s="28" t="inlineStr">
         <is>
-          <t>Linked controls (GT AI RCM v2.1)</t>
+          <t>Linked controls (GT AI Risk Assessment Framework)</t>
         </is>
       </c>
       <c r="J8" s="28" t="inlineStr">
@@ -2095,7 +2095,7 @@
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="29" t="inlineStr">
         <is>
-          <t>PART B  -  AI READINESS &amp; CONTROL MATURITY  (5 domains + GT AI RCM: how well is it managed?)</t>
+          <t>PART B  -  AI READINESS &amp; CONTROL MATURITY  (5 domains + GT AI Risk Assessment Framework controls: how well is it managed?)</t>
         </is>
       </c>
       <c r="C14" s="21" t="n"/>
@@ -3309,7 +3309,7 @@
     </row>
     <row r="4">
       <c r="B4" s="44" t="str">
-        <f>IF(Calc!B21=1,"Framework basis: NSW AI Assessment Framework (inherent risk)  |  ISO/IEC 42001, ISO/IEC 23894, NIST AI RMF  |  EU AI Act, Bahrain PDPL  |  GT AI RCM v2.1 (controls)","ASSESSMENT INCOMPLETE - "&amp;Calc!B20&amp;" of 20 questions answered. Results below are provisional.")</f>
+        <f>IF(Calc!B21=1,"Framework basis: NSW AI Assessment Framework (inherent risk)  |  ISO/IEC 42001, ISO/IEC 23894, NIST AI RMF  |  EU AI Act, Bahrain PDPL  |  GT AI Risk Assessment Framework (controls)","ASSESSMENT INCOMPLETE - "&amp;Calc!B20&amp;" of 20 questions answered. Results below are provisional.")</f>
         <v>ASSESSMENT INCOMPLETE - 0 of 20 questions answered. Results below are provisional.</v>
       </c>
       <c r="M4" s="45" t="n"/>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="G106" s="76" t="inlineStr">
         <is>
-          <t>Lawful basis and notice for AI processing; DPIAs; security; data-subject rights incl. objection to automated processing; cross-border transfer rules for AI services hosted outside Bahrain (RCM PR-1 to PR-6).</t>
+          <t>Lawful basis and notice for AI processing; DPIAs; security; data-subject rights incl. objection to automated processing; cross-border transfer rules for AI services hosted outside Bahrain (controls PR-1 to PR-6).</t>
         </is>
       </c>
       <c r="H106" s="21" t="n"/>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="G107" s="76" t="inlineStr">
         <is>
-          <t>National AI policy pillars (compliance, adoption, awareness, cooperation) and GCC ethics principles - mandatory reference for government entities and good practice for all (RCM GL-1, GL-4, RS-series).</t>
+          <t>National AI policy pillars (compliance, adoption, awareness, cooperation) and GCC ethics principles - mandatory reference for government entities and good practice for all (controls GL-1, GL-4, RS-series).</t>
         </is>
       </c>
       <c r="H107" s="21" t="n"/>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="G108" s="76" t="inlineStr">
         <is>
-          <t>Board oversight, risk management, cyber security, outsourcing and consumer-protection requirements apply to AI; expect model validation for material models and notification of material outsourcing (RCM LC-9, TP-3, AT-3).</t>
+          <t>Board oversight, risk management, cyber security, outsourcing and consumer-protection requirements apply to AI; expect model validation for material models and notification of material outsourcing (controls LC-9, TP-3, AT-3).</t>
         </is>
       </c>
       <c r="H108" s="21" t="n"/>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="G109" s="76" t="inlineStr">
         <is>
-          <t>Extraterritorial reach. Prohibited practices (Art. 5) and AI literacy (Art. 4) apply since Feb 2025; GPAI rules since Aug 2025; transparency (Art. 50) from Aug 2026 (RCM RM-5, GL-4, CO-1, LC-7).</t>
+          <t>Extraterritorial reach. Prohibited practices (Art. 5) and AI literacy (Art. 4) apply since Feb 2025; GPAI rules since Aug 2025; transparency (Art. 50) from Aug 2026 (controls RM-5, GL-4, CO-1, LC-7).</t>
         </is>
       </c>
       <c r="H109" s="21" t="n"/>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="G110" s="76" t="inlineStr">
         <is>
-          <t>Decisions on credit, employment, insurance, essential services etc. may be high-risk: risk management, data governance, logging, human oversight, FRIA and registration (timelines subject to the EU Digital Omnibus outcome) (RCM RO-6).</t>
+          <t>Decisions on credit, employment, insurance, essential services etc. may be high-risk: risk management, data governance, logging, human oversight, FRIA and registration (timelines subject to the EU Digital Omnibus outcome) (controls RO-6).</t>
         </is>
       </c>
       <c r="H110" s="21" t="n"/>
@@ -5458,7 +5458,7 @@
       </c>
       <c r="G111" s="76" t="inlineStr">
         <is>
-          <t>Include in the AI obligations register; align data-transfer, ethics and sector AI requirements across GCC operations (RCM RO-5).</t>
+          <t>Include in the AI obligations register; align data-transfer, ethics and sector AI requirements across GCC operations (controls RO-5).</t>
         </is>
       </c>
       <c r="H111" s="21" t="n"/>
@@ -5484,7 +5484,7 @@
       </c>
       <c r="G112" s="76" t="inlineStr">
         <is>
-          <t>International certifiable standard for AI governance; demonstrates trustworthy AI to clients and regulators. Recommended once readiness reaches 'Repeatable' (RCM AA-2).</t>
+          <t>International certifiable standard for AI governance; demonstrates trustworthy AI to clients and regulators. Recommended once readiness reaches 'Repeatable' (controls AA-2).</t>
         </is>
       </c>
       <c r="H112" s="21" t="n"/>
@@ -5510,7 +5510,7 @@
       </c>
       <c r="G113" s="76" t="inlineStr">
         <is>
-          <t>Proposed standalone AI law (38 articles) with a new regulator and penalties - not yet in force. Maintain horizon scanning (RCM RO-5).</t>
+          <t>Proposed standalone AI law (38 articles) with a new regulator and penalties - not yet in force. Maintain horizon scanning (controls RO-5).</t>
         </is>
       </c>
       <c r="H113" s="21" t="n"/>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="F117" s="65" t="inlineStr">
         <is>
-          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, RCM-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
+          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, framework-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
         </is>
       </c>
       <c r="G117" s="21" t="n"/>
@@ -5777,7 +5777,7 @@
     <row r="131" ht="58" customHeight="1">
       <c r="B131" s="81" t="inlineStr">
         <is>
-          <t>Methodology: Part A (4 questions) derives an inherent-risk tier from the NSW AI Assessment Framework risk factors (AI use, decision impact, data sensitivity, oversight &amp; reversibility). Part B (16 questions) scores readiness 0-100% across 5 domains (AI Governance; AI Risk &amp; Security; Training &amp; Awareness; Strategy &amp; Value; Data &amp; Technology); domain scores are averaged equally into the overall score and mapped to a four-band maturity scale. Exposure combines tier and maturity. Recommendations reference the GT AI RCM v2.1 controls.  Disclaimer: this is a self-assessment based on the responses provided and has not been independently verified by Grant Thornton. It is not an audit, certification or legal opinion.  (c) 2026 Grant Thornton Bahrain. All rights reserved.</t>
+          <t>Methodology: Part A (4 questions) derives an inherent-risk tier from the NSW AI Assessment Framework risk factors (AI use, decision impact, data sensitivity, oversight &amp; reversibility). Part B (16 questions) scores readiness 0-100% across 5 domains (AI Governance; AI Risk &amp; Security; Training &amp; Awareness; Strategy &amp; Value; Data &amp; Technology); domain scores are averaged equally into the overall score and mapped to a four-band maturity scale. Exposure combines tier and maturity. Recommendations reference the controls of the GT AI Risk Assessment Framework.  Disclaimer: this is a self-assessment based on the responses provided and has not been independently verified by Grant Thornton. It is not an audit, certification or legal opinion.  (c) 2026 Grant Thornton Bahrain. All rights reserved.</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
       </c>
       <c r="H4" s="28" t="inlineStr">
         <is>
-          <t>Linked controls (RCM v2.1)</t>
+          <t>Linked controls (GT AI Risk Assessment Framework)</t>
         </is>
       </c>
       <c r="I4" s="28" t="inlineStr">
@@ -7125,12 +7125,12 @@
       <c r="G3" s="21" t="n"/>
       <c r="H3" s="21" t="n"/>
     </row>
-    <row r="4" ht="84" customHeight="1">
+    <row r="4" ht="97" customHeight="1">
       <c r="B4" s="84" t="inlineStr">
         <is>
           <t>1) NSW AI Assessment Framework (AIAF, Digital NSW): lifecycle triggers, inherent-risk questions (AI use, decision impact, data, autonomy / reversibility), Low-Critical risk bands, pattern overrides, oversight pathways and the 8 ethics principles.
 2) GT AI Ready7: the 7 pillars (33 items) are consolidated into 5 domains - AI Governance; AI Risk &amp; Security (Protect AI Systems + Protection from AI Threats, plus AI risk management); Training &amp; Awareness; Strategy &amp; Value; Data &amp; Technology - using the AI Ready7 maturity scale Partial / Informed / Repeatable / Adaptive.
-3) GT AI RCM v2.1: every readiness question is mapped to the controls that evidence it, so results convert directly into a control-remediation plan.</t>
+3) GT AI Risk Assessment Framework: every readiness question is mapped to the controls that evidence it, so results convert directly into a control-remediation plan.</t>
         </is>
       </c>
       <c r="C4" s="21" t="n"/>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="G26" s="28" t="inlineStr">
         <is>
-          <t>GT AI RCM v2.1 controls</t>
+          <t>GT AI Risk Assessment Framework controls</t>
         </is>
       </c>
       <c r="H26" s="28" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Map each obligation to controls and owners using the GT AI RCM; require annual staff acknowledgement.</t>
+          <t>Map each obligation to controls and owners using the GT AI Risk Assessment Framework; require annual staff acknowledgement.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, RCM-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
+          <t>AI governance structure, policies and acceptable use, AI register, guardrails and human-oversight standards, framework-based compliance reviews, ISO/IEC 42001 readiness and internal audit.</t>
         </is>
       </c>
       <c r="D120" t="str">

</xml_diff>